<commit_message>
the shitfuck now quonglebings
</commit_message>
<xml_diff>
--- a/documentation/parts and their channels.xlsx
+++ b/documentation/parts and their channels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Squingle\Desktop\!folders\! d-github\EISS\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9505D36E-7FF2-4519-A2DF-28DAED0E0D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287EE06B-3E1C-4B06-B7D1-AADBDECBE7EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A0965BB0-A002-463F-9819-73939F3991DC}"/>
+    <workbookView xWindow="38280" yWindow="3600" windowWidth="29040" windowHeight="15720" xr2:uid="{A0965BB0-A002-463F-9819-73939F3991DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="96">
   <si>
     <t>Freq:</t>
   </si>
@@ -287,9 +287,6 @@
     <t>old check radar FOVs</t>
   </si>
   <si>
-    <t>gimbal Controls</t>
-  </si>
-  <si>
     <t>enemy transmit 1</t>
   </si>
   <si>
@@ -317,7 +314,16 @@
     <t>missile trans1 index</t>
   </si>
   <si>
-    <t>TWS Dev Version</t>
+    <t>TSD</t>
+  </si>
+  <si>
+    <t>Zoom</t>
+  </si>
+  <si>
+    <t>forward radar ang</t>
+  </si>
+  <si>
+    <t>gimbal controls (might be removed)</t>
   </si>
 </sst>
 </file>
@@ -424,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -435,13 +441,13 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -451,6 +457,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -767,70 +776,98 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AA91CC7-EF17-44C0-8F91-86ED01CBB552}">
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:W71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="28.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="11.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="6.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="6.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="26.85546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="31.5703125" style="1" customWidth="1"/>
-    <col min="8" max="9" width="9.140625" style="1"/>
-    <col min="10" max="10" width="19.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="18.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="1"/>
+    <col min="9" max="9" width="7.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="21" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.5703125" style="1" customWidth="1"/>
     <col min="12" max="13" width="9.140625" style="1"/>
     <col min="14" max="14" width="11.42578125" style="1" customWidth="1"/>
     <col min="15" max="15" width="12.28515625" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="1"/>
+    <col min="16" max="16" width="9.140625" style="1"/>
+    <col min="17" max="17" width="7.42578125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="20.85546875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="17.5703125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="9.140625" style="1"/>
+    <col min="21" max="21" width="7.28515625" style="1" customWidth="1"/>
+    <col min="22" max="22" width="12.140625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="13.42578125" style="1" customWidth="1"/>
+    <col min="24" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="I1" s="6" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="I1" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-    </row>
-    <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="Q1" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+    </row>
+    <row r="2" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6" t="s">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="I2" s="6" t="s">
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="I2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6" t="s">
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="Q2" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="5"/>
+      <c r="U2" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="V2" s="5"/>
+      <c r="W2" s="5"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -840,7 +877,7 @@
       <c r="C3" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="6"/>
+      <c r="D3" s="5"/>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
@@ -859,7 +896,7 @@
       <c r="K3" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="L3" s="6"/>
+      <c r="L3" s="5"/>
       <c r="M3" s="3" t="s">
         <v>0</v>
       </c>
@@ -869,25 +906,44 @@
       <c r="O3" s="3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="T3" s="5"/>
+      <c r="U3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="W3" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="6"/>
+      <c r="D4" s="5"/>
       <c r="E4" s="2">
         <v>1</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>70</v>
       </c>
       <c r="I4" s="2">
@@ -896,55 +952,83 @@
       <c r="J4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="L4" s="6"/>
+      <c r="L4" s="5"/>
       <c r="M4" s="2">
         <v>1</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q4" s="2">
+        <v>1</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="S4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="T4" s="5"/>
+      <c r="U4" s="2">
+        <v>1</v>
+      </c>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="5"/>
       <c r="E5" s="2">
         <v>2</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G5" s="5"/>
+      <c r="G5" s="6"/>
       <c r="I5" s="2">
         <v>2</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K5" s="5"/>
-      <c r="L5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="5"/>
       <c r="M5" s="2">
         <v>2</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
-    </row>
-    <row r="6" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q5" s="2">
+        <v>2</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="S5" s="6"/>
+      <c r="T5" s="5"/>
+      <c r="U5" s="2">
+        <v>2</v>
+      </c>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+    </row>
+    <row r="6" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="5"/>
       <c r="E6" s="2">
         <v>3</v>
       </c>
@@ -960,25 +1044,38 @@
       <c r="J6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K6" s="5"/>
-      <c r="L6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="5"/>
       <c r="M6" s="2">
         <v>3</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
-    </row>
-    <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q6" s="2">
+        <v>3</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="S6" s="6"/>
+      <c r="T6" s="5"/>
+      <c r="U6" s="2">
+        <v>3</v>
+      </c>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+    </row>
+    <row r="7" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="6"/>
+      <c r="D7" s="5"/>
       <c r="E7" s="2">
         <v>4</v>
       </c>
@@ -994,32 +1091,47 @@
       <c r="J7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="L7" s="6"/>
+      <c r="L7" s="5"/>
       <c r="M7" s="2">
         <v>4</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q7" s="2">
+        <v>4</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="S7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="T7" s="5"/>
+      <c r="U7" s="2">
+        <v>4</v>
+      </c>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="5"/>
       <c r="E8" s="2">
         <v>5</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>80</v>
       </c>
       <c r="I8" s="2">
@@ -1028,62 +1140,88 @@
       <c r="J8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K8" s="5"/>
-      <c r="L8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="5"/>
       <c r="M8" s="2">
         <v>5</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q8" s="2">
+        <v>5</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="S8" s="6"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="2">
+        <v>5</v>
+      </c>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="5"/>
       <c r="E9" s="2">
         <v>6</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G9" s="5"/>
+      <c r="G9" s="6"/>
       <c r="I9" s="2">
         <v>6</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K9" s="5"/>
-      <c r="L9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="5"/>
       <c r="M9" s="2">
         <v>6</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-    </row>
-    <row r="10" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q9" s="2">
+        <v>6</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="S9" s="6"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="2">
+        <v>6</v>
+      </c>
+      <c r="V9" s="2"/>
+      <c r="W9" s="2"/>
+    </row>
+    <row r="10" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="6"/>
+      <c r="D10" s="5"/>
       <c r="E10" s="2">
         <v>7</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="6" t="s">
         <v>81</v>
       </c>
       <c r="I10" s="2">
@@ -1092,62 +1230,90 @@
       <c r="J10" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="K10" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="L10" s="6"/>
+      <c r="K10" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="L10" s="5"/>
       <c r="M10" s="2">
         <v>7</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-    </row>
-    <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q10" s="2">
+        <v>7</v>
+      </c>
+      <c r="R10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="S10" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="T10" s="5"/>
+      <c r="U10" s="2">
+        <v>7</v>
+      </c>
+      <c r="V10" s="2"/>
+      <c r="W10" s="2"/>
+    </row>
+    <row r="11" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="5"/>
       <c r="E11" s="2">
         <v>8</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G11" s="5"/>
+      <c r="G11" s="6"/>
       <c r="I11" s="2">
         <v>8</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K11" s="5"/>
-      <c r="L11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="5"/>
       <c r="M11" s="2">
         <v>8</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
-    </row>
-    <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q11" s="2">
+        <v>8</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="S11" s="6"/>
+      <c r="T11" s="5"/>
+      <c r="U11" s="2">
+        <v>8</v>
+      </c>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
+    </row>
+    <row r="12" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="5"/>
       <c r="E12" s="2">
         <v>9</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="6" t="s">
         <v>82</v>
       </c>
       <c r="I12" s="2">
@@ -1156,65 +1322,93 @@
       <c r="J12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="K12" s="5"/>
-      <c r="L12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="5"/>
       <c r="M12" s="2">
         <v>9</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
-    </row>
-    <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q12" s="2">
+        <v>9</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="S12" s="6"/>
+      <c r="T12" s="5"/>
+      <c r="U12" s="2">
+        <v>9</v>
+      </c>
+      <c r="V12" s="2"/>
+      <c r="W12" s="2"/>
+    </row>
+    <row r="13" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="6"/>
+      <c r="D13" s="5"/>
       <c r="E13" s="2">
         <v>10</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G13" s="5"/>
+      <c r="G13" s="6"/>
       <c r="I13" s="2">
         <v>10</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="K13" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="L13" s="6"/>
+      <c r="K13" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="L13" s="5"/>
       <c r="M13" s="2">
         <v>10</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q13" s="2">
+        <v>10</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="S13" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="T13" s="5"/>
+      <c r="U13" s="2">
+        <v>10</v>
+      </c>
+      <c r="V13" s="2"/>
+      <c r="W13" s="2"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="5"/>
       <c r="E14" s="2">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>83</v>
+      <c r="G14" s="6" t="s">
+        <v>95</v>
       </c>
       <c r="I14" s="2">
         <v>11</v>
@@ -1222,95 +1416,136 @@
       <c r="J14" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="K14" s="5"/>
-      <c r="L14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="5"/>
       <c r="M14" s="2">
         <v>11</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q14" s="2">
+        <v>11</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="S14" s="6"/>
+      <c r="T14" s="5"/>
+      <c r="U14" s="2">
+        <v>11</v>
+      </c>
+      <c r="V14" s="2"/>
+      <c r="W14" s="2"/>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="6"/>
+      <c r="D15" s="5"/>
       <c r="E15" s="2">
         <v>12</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G15" s="5"/>
+      <c r="G15" s="6"/>
       <c r="I15" s="2">
         <v>12</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="K15" s="5"/>
-      <c r="L15" s="6"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="5"/>
       <c r="M15" s="2">
         <v>12</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q15" s="2">
+        <v>12</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="S15" s="6"/>
+      <c r="T15" s="5"/>
+      <c r="U15" s="2">
+        <v>12</v>
+      </c>
+      <c r="V15" s="2"/>
+      <c r="W15" s="2"/>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="5"/>
       <c r="E16" s="2">
         <v>13</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G16" s="5"/>
+      <c r="G16" s="6"/>
       <c r="I16" s="2">
         <v>13</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="K16" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="L16" s="6"/>
+      <c r="K16" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="L16" s="5"/>
       <c r="M16" s="2">
         <v>13</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q16" s="2">
+        <v>13</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="S16" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="T16" s="5"/>
+      <c r="U16" s="2">
+        <v>13</v>
+      </c>
+      <c r="V16" s="2"/>
+      <c r="W16" s="2"/>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="5"/>
       <c r="E17" s="2">
         <v>14</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G17" s="5" t="s">
-        <v>84</v>
+      <c r="G17" s="6" t="s">
+        <v>83</v>
       </c>
       <c r="I17" s="2">
         <v>14</v>
@@ -1318,95 +1553,136 @@
       <c r="J17" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="K17" s="5"/>
-      <c r="L17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="5"/>
       <c r="M17" s="2">
         <v>14</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q17" s="2">
+        <v>14</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="S17" s="6"/>
+      <c r="T17" s="5"/>
+      <c r="U17" s="2">
+        <v>14</v>
+      </c>
+      <c r="V17" s="2"/>
+      <c r="W17" s="2"/>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="6"/>
+      <c r="D18" s="5"/>
       <c r="E18" s="2">
         <v>15</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G18" s="5"/>
+      <c r="G18" s="6"/>
       <c r="I18" s="2">
         <v>15</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K18" s="5"/>
-      <c r="L18" s="6"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="5"/>
       <c r="M18" s="2">
         <v>15</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q18" s="2">
+        <v>15</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="S18" s="6"/>
+      <c r="T18" s="5"/>
+      <c r="U18" s="2">
+        <v>15</v>
+      </c>
+      <c r="V18" s="2"/>
+      <c r="W18" s="2"/>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="5"/>
       <c r="E19" s="2">
         <v>16</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="G19" s="5"/>
+      <c r="G19" s="6"/>
       <c r="I19" s="2">
         <v>16</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K19" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="L19" s="6"/>
+      <c r="K19" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="L19" s="5"/>
       <c r="M19" s="2">
         <v>16</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q19" s="2">
+        <v>16</v>
+      </c>
+      <c r="R19" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="S19" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="T19" s="5"/>
+      <c r="U19" s="2">
+        <v>16</v>
+      </c>
+      <c r="V19" s="2"/>
+      <c r="W19" s="2"/>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="5"/>
       <c r="E20" s="2">
         <v>17</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G20" s="5" t="s">
-        <v>85</v>
+      <c r="G20" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="I20" s="2">
         <v>17</v>
@@ -1414,62 +1690,88 @@
       <c r="J20" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="K20" s="5"/>
-      <c r="L20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="5"/>
       <c r="M20" s="2">
         <v>17</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q20" s="2">
+        <v>17</v>
+      </c>
+      <c r="R20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="S20" s="6"/>
+      <c r="T20" s="5"/>
+      <c r="U20" s="2">
+        <v>17</v>
+      </c>
+      <c r="V20" s="2"/>
+      <c r="W20" s="2"/>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D21" s="6"/>
+      <c r="D21" s="5"/>
       <c r="E21" s="2">
         <v>18</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G21" s="5"/>
+      <c r="G21" s="6"/>
       <c r="I21" s="2">
         <v>18</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="K21" s="5"/>
-      <c r="L21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="5"/>
       <c r="M21" s="2">
         <v>18</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
-    </row>
-    <row r="22" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q21" s="2">
+        <v>18</v>
+      </c>
+      <c r="R21" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="S21" s="6"/>
+      <c r="T21" s="5"/>
+      <c r="U21" s="2">
+        <v>18</v>
+      </c>
+      <c r="V21" s="2"/>
+      <c r="W21" s="2"/>
+    </row>
+    <row r="22" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="5"/>
       <c r="E22" s="2">
         <v>19</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="G22" s="5"/>
+      <c r="G22" s="6"/>
       <c r="I22" s="2">
         <v>19</v>
       </c>
@@ -1479,30 +1781,45 @@
       <c r="K22" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="L22" s="6"/>
+      <c r="L22" s="5"/>
       <c r="M22" s="2">
         <v>19</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
-    </row>
-    <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q22" s="2">
+        <v>19</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="S22" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T22" s="5"/>
+      <c r="U22" s="2">
+        <v>19</v>
+      </c>
+      <c r="V22" s="2"/>
+      <c r="W22" s="2"/>
+    </row>
+    <row r="23" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="5"/>
-      <c r="D23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="5"/>
       <c r="E23" s="2">
         <v>20</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>86</v>
+      <c r="G23" s="6" t="s">
+        <v>85</v>
       </c>
       <c r="I23" s="2">
         <v>20</v>
@@ -1511,31 +1828,44 @@
         <v>73</v>
       </c>
       <c r="K23" s="8"/>
-      <c r="L23" s="6"/>
+      <c r="L23" s="5"/>
       <c r="M23" s="2">
         <v>20</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
-    </row>
-    <row r="24" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q23" s="2">
+        <v>20</v>
+      </c>
+      <c r="R23" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="S23" s="8"/>
+      <c r="T23" s="5"/>
+      <c r="U23" s="2">
+        <v>20</v>
+      </c>
+      <c r="V23" s="2"/>
+      <c r="W23" s="2"/>
+    </row>
+    <row r="24" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="6"/>
+      <c r="D24" s="5"/>
       <c r="E24" s="2">
         <v>21</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G24" s="5"/>
+      <c r="G24" s="6"/>
       <c r="I24" s="2">
         <v>21</v>
       </c>
@@ -1543,155 +1873,222 @@
         <v>74</v>
       </c>
       <c r="K24" s="8"/>
-      <c r="L24" s="6"/>
+      <c r="L24" s="5"/>
       <c r="M24" s="2">
         <v>21</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q24" s="2">
+        <v>21</v>
+      </c>
+      <c r="R24" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="S24" s="8"/>
+      <c r="T24" s="5"/>
+      <c r="U24" s="2">
+        <v>21</v>
+      </c>
+      <c r="V24" s="2"/>
+      <c r="W24" s="2"/>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="5"/>
-      <c r="D25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="5"/>
       <c r="E25" s="2">
         <v>22</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G25" s="5"/>
+      <c r="G25" s="6"/>
       <c r="I25" s="2">
         <v>22</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K25" s="9"/>
-      <c r="L25" s="6"/>
+      <c r="L25" s="5"/>
       <c r="M25" s="2">
         <v>22</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q25" s="2">
+        <v>22</v>
+      </c>
+      <c r="R25" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="S25" s="9"/>
+      <c r="T25" s="5"/>
+      <c r="U25" s="2">
+        <v>22</v>
+      </c>
+      <c r="V25" s="2"/>
+      <c r="W25" s="2"/>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="5"/>
-      <c r="D26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="5"/>
       <c r="E26" s="2">
         <v>23</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="G26" s="5" t="s">
-        <v>87</v>
+      <c r="G26" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="I26" s="2">
         <v>23</v>
       </c>
       <c r="J26" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K26" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="L26" s="6"/>
+      <c r="L26" s="5"/>
       <c r="M26" s="2">
         <v>23</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q26" s="2">
+        <v>23</v>
+      </c>
+      <c r="R26" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="S26" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="T26" s="5"/>
+      <c r="U26" s="2">
+        <v>23</v>
+      </c>
+      <c r="V26" s="2"/>
+      <c r="W26" s="2"/>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="6"/>
+      <c r="D27" s="5"/>
       <c r="E27" s="2">
         <v>24</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G27" s="5"/>
+      <c r="G27" s="6"/>
       <c r="I27" s="2">
         <v>24</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K27" s="2"/>
-      <c r="L27" s="6"/>
+      <c r="L27" s="5"/>
       <c r="M27" s="2">
         <v>24</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
-    </row>
-    <row r="28" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q27" s="2">
+        <v>24</v>
+      </c>
+      <c r="R27" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="S27" s="8"/>
+      <c r="T27" s="5"/>
+      <c r="U27" s="2">
+        <v>24</v>
+      </c>
+      <c r="V27" s="2"/>
+      <c r="W27" s="2"/>
+    </row>
+    <row r="28" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="5"/>
-      <c r="D28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="5"/>
       <c r="E28" s="2">
         <v>25</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G28" s="5"/>
+      <c r="G28" s="6"/>
       <c r="I28" s="2">
         <v>25</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K28" s="2"/>
-      <c r="L28" s="6"/>
+      <c r="L28" s="5"/>
       <c r="M28" s="2">
         <v>25</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
-    </row>
-    <row r="29" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q28" s="2">
+        <v>25</v>
+      </c>
+      <c r="R28" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="S28" s="9"/>
+      <c r="T28" s="5"/>
+      <c r="U28" s="2">
+        <v>25</v>
+      </c>
+      <c r="V28" s="2"/>
+      <c r="W28" s="2"/>
+    </row>
+    <row r="29" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C29" s="5"/>
-      <c r="D29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="5"/>
       <c r="E29" s="2">
         <v>26</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G29" s="5" t="s">
+      <c r="G29" s="6" t="s">
         <v>79</v>
       </c>
       <c r="I29" s="2">
@@ -1699,100 +2096,148 @@
       </c>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
-      <c r="L29" s="6"/>
+      <c r="L29" s="5"/>
       <c r="M29" s="2">
         <v>26</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
-    </row>
-    <row r="30" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q29" s="2">
+        <v>26</v>
+      </c>
+      <c r="R29" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="S29" s="2"/>
+      <c r="T29" s="5"/>
+      <c r="U29" s="2">
+        <v>26</v>
+      </c>
+      <c r="V29" s="2"/>
+      <c r="W29" s="2"/>
+    </row>
+    <row r="30" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D30" s="6"/>
+      <c r="D30" s="5"/>
       <c r="E30" s="2">
         <v>27</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G30" s="5"/>
+      <c r="G30" s="6"/>
       <c r="I30" s="2">
         <v>27</v>
       </c>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
-      <c r="L30" s="6"/>
+      <c r="L30" s="5"/>
       <c r="M30" s="2">
         <v>27</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
-    </row>
-    <row r="31" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q30" s="2">
+        <v>27</v>
+      </c>
+      <c r="R30" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="S30" s="2"/>
+      <c r="T30" s="5"/>
+      <c r="U30" s="2">
+        <v>27</v>
+      </c>
+      <c r="V30" s="2"/>
+      <c r="W30" s="2"/>
+    </row>
+    <row r="31" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C31" s="5"/>
-      <c r="D31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="5"/>
       <c r="E31" s="2">
         <v>28</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G31" s="5"/>
+      <c r="G31" s="6"/>
       <c r="I31" s="2">
         <v>28</v>
       </c>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
-      <c r="L31" s="6"/>
+      <c r="L31" s="5"/>
       <c r="M31" s="2">
         <v>28</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q31" s="2">
+        <v>28</v>
+      </c>
+      <c r="R31" s="2"/>
+      <c r="S31" s="2"/>
+      <c r="T31" s="5"/>
+      <c r="U31" s="2">
+        <v>28</v>
+      </c>
+      <c r="V31" s="2"/>
+      <c r="W31" s="2"/>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="5"/>
-      <c r="D32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="5"/>
       <c r="E32" s="2">
         <v>29</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G32" s="5"/>
+        <v>91</v>
+      </c>
+      <c r="G32" s="6"/>
       <c r="I32" s="2">
         <v>29</v>
       </c>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
-      <c r="L32" s="6"/>
+      <c r="L32" s="5"/>
       <c r="M32" s="2">
         <v>29</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
-    </row>
-    <row r="33" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q32" s="2">
+        <v>29</v>
+      </c>
+      <c r="R32" s="2"/>
+      <c r="S32" s="2"/>
+      <c r="T32" s="5"/>
+      <c r="U32" s="2">
+        <v>29</v>
+      </c>
+      <c r="V32" s="2"/>
+      <c r="W32" s="2"/>
+    </row>
+    <row r="33" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>30</v>
       </c>
@@ -1802,632 +2247,315 @@
       <c r="C33" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D33" s="6"/>
+      <c r="D33" s="5"/>
       <c r="E33" s="2">
         <v>30</v>
       </c>
       <c r="F33" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G33" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>91</v>
       </c>
       <c r="I33" s="2">
         <v>30</v>
       </c>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
-      <c r="L33" s="6"/>
+      <c r="L33" s="5"/>
       <c r="M33" s="2">
         <v>30</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
-    </row>
-    <row r="34" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q33" s="2">
+        <v>30</v>
+      </c>
+      <c r="R33" s="2"/>
+      <c r="S33" s="2"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="2">
+        <v>30</v>
+      </c>
+      <c r="V33" s="2"/>
+      <c r="W33" s="2"/>
+    </row>
+    <row r="34" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>31</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D34" s="6"/>
+      <c r="D34" s="5"/>
       <c r="E34" s="2">
         <v>31</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G34" s="5"/>
+        <v>87</v>
+      </c>
+      <c r="G34" s="6"/>
       <c r="I34" s="2">
         <v>31</v>
       </c>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
-      <c r="L34" s="6"/>
+      <c r="L34" s="5"/>
       <c r="M34" s="2">
         <v>31</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
-    </row>
-    <row r="35" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q34" s="2">
+        <v>31</v>
+      </c>
+      <c r="R34" s="2"/>
+      <c r="S34" s="2"/>
+      <c r="T34" s="5"/>
+      <c r="U34" s="2">
+        <v>31</v>
+      </c>
+      <c r="V34" s="2"/>
+      <c r="W34" s="2"/>
+    </row>
+    <row r="35" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>32</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="5"/>
-      <c r="D35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="5"/>
       <c r="E35" s="2">
         <v>32</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G35" s="5"/>
+        <v>88</v>
+      </c>
+      <c r="G35" s="6"/>
       <c r="I35" s="2">
         <v>32</v>
       </c>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
-      <c r="L35" s="6"/>
+      <c r="L35" s="5"/>
       <c r="M35" s="2">
         <v>32</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B38" s="6"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D39" s="6"/>
-      <c r="E39" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="G39" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
-        <v>1</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D40" s="6"/>
-      <c r="E40" s="2">
-        <v>1</v>
-      </c>
-      <c r="F40" s="2"/>
+      <c r="Q35" s="2">
+        <v>32</v>
+      </c>
+      <c r="R35" s="2"/>
+      <c r="S35" s="2"/>
+      <c r="T35" s="5"/>
+      <c r="U35" s="2">
+        <v>32</v>
+      </c>
+      <c r="V35" s="2"/>
+      <c r="W35" s="2"/>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A37" s="10"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A38" s="10"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="D39" s="10"/>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
       <c r="G40" s="4"/>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
-        <v>2</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C41" s="5"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="2">
-        <v>2</v>
-      </c>
-      <c r="F41" s="2"/>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
       <c r="G41" s="4"/>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
-        <v>3</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C42" s="5"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="2">
-        <v>3</v>
-      </c>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
-        <v>4</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D43" s="6"/>
-      <c r="E43" s="2">
-        <v>4</v>
-      </c>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
-        <v>5</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="6"/>
-      <c r="E44" s="2">
-        <v>5</v>
-      </c>
-      <c r="F44" s="2"/>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
       <c r="G44" s="4"/>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
-        <v>6</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C45" s="5"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="2">
-        <v>6</v>
-      </c>
-      <c r="F45" s="2"/>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
       <c r="G45" s="4"/>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
-        <v>7</v>
-      </c>
-      <c r="B46" s="2"/>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C46" s="4"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="2">
-        <v>7</v>
-      </c>
-      <c r="F46" s="2"/>
+      <c r="D46" s="10"/>
       <c r="G46" s="4"/>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A47" s="2">
-        <v>8</v>
-      </c>
-      <c r="B47" s="2"/>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C47" s="4"/>
-      <c r="D47" s="6"/>
-      <c r="E47" s="2">
-        <v>8</v>
-      </c>
-      <c r="F47" s="2"/>
+      <c r="D47" s="10"/>
       <c r="G47" s="4"/>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="2">
-        <v>9</v>
-      </c>
-      <c r="B48" s="2"/>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C48" s="4"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="2">
-        <v>9</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G48" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
-        <v>10</v>
-      </c>
-      <c r="B49" s="2"/>
+      <c r="D48" s="10"/>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C49" s="4"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="2">
-        <v>10</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G49" s="5"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="2">
-        <v>11</v>
-      </c>
-      <c r="B50" s="2"/>
+      <c r="D49" s="10"/>
+      <c r="G49" s="10"/>
+    </row>
+    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C50" s="4"/>
-      <c r="D50" s="6"/>
-      <c r="E50" s="2">
-        <v>11</v>
-      </c>
-      <c r="F50" s="2"/>
+      <c r="D50" s="10"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="2">
-        <v>12</v>
-      </c>
-      <c r="B51" s="2"/>
+    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C51" s="4"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="2">
-        <v>12</v>
-      </c>
-      <c r="F51" s="2"/>
+      <c r="D51" s="10"/>
       <c r="G51" s="4"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="2">
-        <v>13</v>
-      </c>
-      <c r="B52" s="2"/>
+    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C52" s="4"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="2">
-        <v>13</v>
-      </c>
-      <c r="F52" s="2"/>
+      <c r="D52" s="10"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="2">
-        <v>14</v>
-      </c>
-      <c r="B53" s="2"/>
+    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C53" s="4"/>
-      <c r="D53" s="6"/>
-      <c r="E53" s="2">
-        <v>14</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G53" s="5" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="2">
-        <v>15</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D54" s="6"/>
-      <c r="E54" s="2">
-        <v>15</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G54" s="5"/>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="2">
-        <v>16</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C55" s="5"/>
-      <c r="D55" s="6"/>
-      <c r="E55" s="2">
-        <v>16</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G55" s="5"/>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="2">
-        <v>17</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C56" s="5"/>
-      <c r="D56" s="6"/>
-      <c r="E56" s="2">
-        <v>17</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G56" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="2">
-        <v>18</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D57" s="6"/>
-      <c r="E57" s="2">
-        <v>18</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G57" s="5"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="2">
-        <v>19</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="6"/>
-      <c r="E58" s="2">
-        <v>19</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G58" s="5"/>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="2">
-        <v>20</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C59" s="5"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="2">
-        <v>20</v>
-      </c>
-      <c r="F59" s="2"/>
+      <c r="D53" s="10"/>
+      <c r="G53" s="10"/>
+    </row>
+    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C54" s="10"/>
+      <c r="D54" s="10"/>
+      <c r="G54" s="10"/>
+    </row>
+    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C55" s="10"/>
+      <c r="D55" s="10"/>
+      <c r="G55" s="10"/>
+    </row>
+    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C56" s="10"/>
+      <c r="D56" s="10"/>
+      <c r="G56" s="10"/>
+    </row>
+    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C57" s="10"/>
+      <c r="D57" s="10"/>
+      <c r="G57" s="10"/>
+    </row>
+    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C58" s="10"/>
+      <c r="D58" s="10"/>
+      <c r="G58" s="10"/>
+    </row>
+    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C59" s="10"/>
+      <c r="D59" s="10"/>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="2">
-        <v>21</v>
-      </c>
-      <c r="B60" s="2"/>
+    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C60" s="4"/>
-      <c r="D60" s="6"/>
-      <c r="E60" s="2">
-        <v>21</v>
-      </c>
-      <c r="F60" s="2"/>
+      <c r="D60" s="10"/>
       <c r="G60" s="4"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="2">
-        <v>22</v>
-      </c>
-      <c r="B61" s="2"/>
+    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C61" s="4"/>
-      <c r="D61" s="6"/>
-      <c r="E61" s="2">
-        <v>22</v>
-      </c>
-      <c r="F61" s="2"/>
+      <c r="D61" s="10"/>
       <c r="G61" s="4"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="2">
-        <v>23</v>
-      </c>
-      <c r="B62" s="2"/>
+    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C62" s="4"/>
-      <c r="D62" s="6"/>
-      <c r="E62" s="2">
-        <v>23</v>
-      </c>
-      <c r="F62" s="2"/>
+      <c r="D62" s="10"/>
       <c r="G62" s="4"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="2">
-        <v>24</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D63" s="6"/>
-      <c r="E63" s="2">
-        <v>24</v>
-      </c>
-      <c r="F63" s="2"/>
+    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C63" s="10"/>
+      <c r="D63" s="10"/>
       <c r="G63" s="4"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="2">
-        <v>25</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C64" s="5"/>
-      <c r="D64" s="6"/>
-      <c r="E64" s="2">
-        <v>25</v>
-      </c>
-      <c r="F64" s="2"/>
+    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C64" s="10"/>
+      <c r="D64" s="10"/>
       <c r="G64" s="4"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="2">
-        <v>26</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C65" s="5"/>
-      <c r="D65" s="6"/>
-      <c r="E65" s="2">
-        <v>26</v>
-      </c>
-      <c r="F65" s="2"/>
+    <row r="65" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C65" s="10"/>
+      <c r="D65" s="10"/>
       <c r="G65" s="4"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="2">
-        <v>27</v>
-      </c>
-      <c r="B66" s="2"/>
+    <row r="66" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C66" s="4"/>
-      <c r="D66" s="6"/>
-      <c r="E66" s="2">
-        <v>27</v>
-      </c>
-      <c r="F66" s="2"/>
+      <c r="D66" s="10"/>
       <c r="G66" s="4"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="2">
-        <v>28</v>
-      </c>
-      <c r="B67" s="2"/>
+    <row r="67" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C67" s="4"/>
-      <c r="D67" s="6"/>
-      <c r="E67" s="2">
-        <v>28</v>
-      </c>
-      <c r="F67" s="2"/>
+      <c r="D67" s="10"/>
       <c r="G67" s="4"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="2">
-        <v>29</v>
-      </c>
-      <c r="B68" s="2"/>
+    <row r="68" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C68" s="4"/>
-      <c r="D68" s="6"/>
-      <c r="E68" s="2">
-        <v>29</v>
-      </c>
-      <c r="F68" s="2"/>
+      <c r="D68" s="10"/>
       <c r="G68" s="4"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="2">
-        <v>30</v>
-      </c>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="6"/>
-      <c r="E69" s="2">
-        <v>30</v>
-      </c>
-      <c r="F69" s="2"/>
+    <row r="69" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D69" s="10"/>
       <c r="G69" s="4"/>
     </row>
-    <row r="70" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A70" s="2">
-        <v>31</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D70" s="6"/>
-      <c r="E70" s="2">
-        <v>31</v>
-      </c>
-      <c r="F70" s="2"/>
+    <row r="70" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C70" s="4"/>
+      <c r="D70" s="10"/>
       <c r="G70" s="4"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="2">
-        <v>32</v>
-      </c>
-      <c r="B71" s="2"/>
+    <row r="71" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C71" s="4"/>
-      <c r="D71" s="6"/>
-      <c r="E71" s="2">
-        <v>32</v>
-      </c>
-      <c r="F71" s="2"/>
+      <c r="D71" s="10"/>
       <c r="G71" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="49">
-    <mergeCell ref="G56:G58"/>
-    <mergeCell ref="C57:C59"/>
-    <mergeCell ref="C63:C65"/>
-    <mergeCell ref="A37:G37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:D71"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="G48:G49"/>
-    <mergeCell ref="G53:G55"/>
-    <mergeCell ref="C54:C56"/>
-    <mergeCell ref="K19:K21"/>
-    <mergeCell ref="K16:K18"/>
-    <mergeCell ref="G20:G22"/>
-    <mergeCell ref="G23:G25"/>
-    <mergeCell ref="G26:G28"/>
+  <mergeCells count="61">
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="D2:D35"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="C27:C29"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="C21:C23"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="C15:C17"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="G4:G5"/>
     <mergeCell ref="I1:O1"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="L2:L35"/>
@@ -2444,22 +2572,35 @@
     <mergeCell ref="K10:K12"/>
     <mergeCell ref="K4:K6"/>
     <mergeCell ref="K7:K9"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="D2:D35"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="C30:C32"/>
-    <mergeCell ref="C27:C29"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="C21:C23"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="C15:C17"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="K19:K21"/>
+    <mergeCell ref="K16:K18"/>
+    <mergeCell ref="G20:G22"/>
+    <mergeCell ref="G23:G25"/>
+    <mergeCell ref="G26:G28"/>
+    <mergeCell ref="G56:G58"/>
+    <mergeCell ref="C57:C59"/>
+    <mergeCell ref="C63:C65"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:D71"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="G48:G49"/>
+    <mergeCell ref="G53:G55"/>
+    <mergeCell ref="C54:C56"/>
+    <mergeCell ref="Q1:W1"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="T2:T35"/>
+    <mergeCell ref="U2:W2"/>
+    <mergeCell ref="S4:S6"/>
+    <mergeCell ref="S7:S9"/>
+    <mergeCell ref="S10:S12"/>
+    <mergeCell ref="S13:S15"/>
+    <mergeCell ref="S16:S18"/>
+    <mergeCell ref="S19:S21"/>
+    <mergeCell ref="S22:S25"/>
+    <mergeCell ref="S26:S28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update parts and their channels.xlsx
</commit_message>
<xml_diff>
--- a/documentation/parts and their channels.xlsx
+++ b/documentation/parts and their channels.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Squingle\Desktop\!folders\! d-github\EISS\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eafacaeacfb09265/Skrivebord/! github/EISS/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D64F8E07-AE90-466C-91F2-FB95F6DDF4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{D64F8E07-AE90-466C-91F2-FB95F6DDF4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B2540F9-C9C2-41FE-B30A-D0FC8812804C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A0965BB0-A002-463F-9819-73939F3991DC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A0965BB0-A002-463F-9819-73939F3991DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -585,13 +585,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -930,98 +930,98 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AA91CC7-EF17-44C0-8F91-86ED01CBB552}">
   <dimension ref="A1:AF71"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="3.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="29.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="31.5703125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" style="1"/>
-    <col min="9" max="9" width="7.85546875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="28.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="18.5703125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="3.42578125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" style="1"/>
-    <col min="14" max="14" width="11.42578125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="12.28515625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="1"/>
-    <col min="17" max="17" width="7.42578125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="3.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="31.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" style="1"/>
+    <col min="9" max="9" width="7.88671875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="28.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.5546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="3.44140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9.109375" style="1"/>
+    <col min="14" max="14" width="11.44140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="12.33203125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="9.109375" style="1"/>
+    <col min="17" max="17" width="7.44140625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.44140625" style="1" customWidth="1"/>
     <col min="19" max="19" width="8" style="1" customWidth="1"/>
-    <col min="20" max="20" width="7.7109375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="7.6640625" style="1" customWidth="1"/>
     <col min="21" max="21" width="12" style="1" customWidth="1"/>
-    <col min="22" max="22" width="12.140625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="13.42578125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="9.140625" style="1"/>
-    <col min="25" max="25" width="6.85546875" style="1" customWidth="1"/>
-    <col min="26" max="26" width="22.85546875" style="1" customWidth="1"/>
-    <col min="27" max="27" width="19.42578125" style="1" customWidth="1"/>
-    <col min="28" max="28" width="2.7109375" style="1" customWidth="1"/>
-    <col min="29" max="29" width="17.5703125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="16.42578125" style="1" customWidth="1"/>
-    <col min="31" max="31" width="15.42578125" style="1" customWidth="1"/>
-    <col min="32" max="16384" width="9.140625" style="1"/>
+    <col min="22" max="22" width="12.109375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="13.44140625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="9.109375" style="1"/>
+    <col min="25" max="25" width="6.88671875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="22.88671875" style="1" customWidth="1"/>
+    <col min="27" max="27" width="19.44140625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="2.6640625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="17.5546875" style="1" customWidth="1"/>
+    <col min="30" max="30" width="16.44140625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="15.44140625" style="1" customWidth="1"/>
+    <col min="32" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
       <c r="H1" s="17"/>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8" t="s">
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8"/>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
       <c r="X1" s="7"/>
-      <c r="AF1" s="8"/>
-    </row>
-    <row r="2" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="AF1" s="10"/>
+    </row>
+    <row r="2" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10" t="s">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
       <c r="H2" s="17"/>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10" t="s">
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="10"/>
       <c r="Q2" s="1" t="s">
         <v>114</v>
       </c>
@@ -1035,9 +1035,9 @@
         <v>113</v>
       </c>
       <c r="X2" s="7"/>
-      <c r="AF2" s="8"/>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF2" s="10"/>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1047,7 +1047,7 @@
       <c r="C3" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="10"/>
+      <c r="D3" s="8"/>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1067,7 +1067,7 @@
       <c r="K3" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="L3" s="10"/>
+      <c r="L3" s="8"/>
       <c r="M3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1077,7 +1077,7 @@
       <c r="O3" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="P3" s="8"/>
+      <c r="P3" s="10"/>
       <c r="Q3" s="1" t="s">
         <v>115</v>
       </c>
@@ -1094,9 +1094,9 @@
         <v>119</v>
       </c>
       <c r="X3" s="7"/>
-      <c r="AF3" s="8"/>
-    </row>
-    <row r="4" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF3" s="10"/>
+    </row>
+    <row r="4" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -1106,7 +1106,7 @@
       <c r="C4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="10"/>
+      <c r="D4" s="8"/>
       <c r="E4" s="2">
         <v>1</v>
       </c>
@@ -1126,13 +1126,13 @@
       <c r="K4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="L4" s="10"/>
+      <c r="L4" s="8"/>
       <c r="M4" s="2">
         <v>1</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
-      <c r="P4" s="8"/>
+      <c r="P4" s="10"/>
       <c r="Q4" s="5" t="b">
         <v>1</v>
       </c>
@@ -1149,9 +1149,9 @@
         <v>1</v>
       </c>
       <c r="X4" s="7"/>
-      <c r="AF4" s="8"/>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF4" s="10"/>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>2</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="9"/>
-      <c r="D5" s="10"/>
+      <c r="D5" s="8"/>
       <c r="E5" s="2">
         <v>2</v>
       </c>
@@ -1175,13 +1175,13 @@
         <v>3</v>
       </c>
       <c r="K5" s="9"/>
-      <c r="L5" s="10"/>
+      <c r="L5" s="8"/>
       <c r="M5" s="2">
         <v>2</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
-      <c r="P5" s="8"/>
+      <c r="P5" s="10"/>
       <c r="Q5" s="5" t="b">
         <v>1</v>
       </c>
@@ -1198,9 +1198,9 @@
         <v>2</v>
       </c>
       <c r="X5" s="7"/>
-      <c r="AF5" s="8"/>
-    </row>
-    <row r="6" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF5" s="10"/>
+    </row>
+    <row r="6" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>3</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="9"/>
-      <c r="D6" s="10"/>
+      <c r="D6" s="8"/>
       <c r="E6" s="2">
         <v>3</v>
       </c>
@@ -1226,13 +1226,13 @@
         <v>4</v>
       </c>
       <c r="K6" s="9"/>
-      <c r="L6" s="10"/>
+      <c r="L6" s="8"/>
       <c r="M6" s="2">
         <v>3</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
-      <c r="P6" s="8"/>
+      <c r="P6" s="10"/>
       <c r="Q6" s="5" t="b">
         <v>1</v>
       </c>
@@ -1249,9 +1249,9 @@
         <v>3</v>
       </c>
       <c r="X6" s="7"/>
-      <c r="AF6" s="8"/>
-    </row>
-    <row r="7" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF6" s="10"/>
+    </row>
+    <row r="7" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>4</v>
       </c>
@@ -1261,7 +1261,7 @@
       <c r="C7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="10"/>
+      <c r="D7" s="8"/>
       <c r="E7" s="2">
         <v>4</v>
       </c>
@@ -1281,13 +1281,13 @@
       <c r="K7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L7" s="10"/>
+      <c r="L7" s="8"/>
       <c r="M7" s="2">
         <v>4</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
-      <c r="P7" s="8"/>
+      <c r="P7" s="10"/>
       <c r="Q7" s="5" t="b">
         <v>1</v>
       </c>
@@ -1304,9 +1304,9 @@
         <v>4</v>
       </c>
       <c r="X7" s="7"/>
-      <c r="AF7" s="8"/>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF7" s="10"/>
+    </row>
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>5</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="9"/>
-      <c r="D8" s="10"/>
+      <c r="D8" s="8"/>
       <c r="E8" s="2">
         <v>5</v>
       </c>
@@ -1332,13 +1332,13 @@
         <v>6</v>
       </c>
       <c r="K8" s="9"/>
-      <c r="L8" s="10"/>
+      <c r="L8" s="8"/>
       <c r="M8" s="2">
         <v>5</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
-      <c r="P8" s="8"/>
+      <c r="P8" s="10"/>
       <c r="Q8" s="5" t="b">
         <v>1</v>
       </c>
@@ -1355,9 +1355,9 @@
         <v>5</v>
       </c>
       <c r="X8" s="7"/>
-      <c r="AF8" s="8"/>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF8" s="10"/>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>6</v>
       </c>
@@ -1365,7 +1365,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="9"/>
-      <c r="D9" s="10"/>
+      <c r="D9" s="8"/>
       <c r="E9" s="2">
         <v>6</v>
       </c>
@@ -1381,13 +1381,13 @@
         <v>7</v>
       </c>
       <c r="K9" s="9"/>
-      <c r="L9" s="10"/>
+      <c r="L9" s="8"/>
       <c r="M9" s="2">
         <v>6</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-      <c r="P9" s="8"/>
+      <c r="P9" s="10"/>
       <c r="Q9" s="5" t="b">
         <v>1</v>
       </c>
@@ -1404,9 +1404,9 @@
         <v>6</v>
       </c>
       <c r="X9" s="7"/>
-      <c r="AF9" s="8"/>
-    </row>
-    <row r="10" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF9" s="10"/>
+    </row>
+    <row r="10" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>7</v>
       </c>
@@ -1416,7 +1416,7 @@
       <c r="C10" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="10"/>
+      <c r="D10" s="8"/>
       <c r="E10" s="2">
         <v>7</v>
       </c>
@@ -1436,13 +1436,13 @@
       <c r="K10" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="L10" s="10"/>
+      <c r="L10" s="8"/>
       <c r="M10" s="2">
         <v>7</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-      <c r="P10" s="8"/>
+      <c r="P10" s="10"/>
       <c r="Q10" s="5" t="b">
         <v>1</v>
       </c>
@@ -1459,9 +1459,9 @@
         <v>7</v>
       </c>
       <c r="X10" s="7"/>
-      <c r="AF10" s="8"/>
-    </row>
-    <row r="11" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF10" s="10"/>
+    </row>
+    <row r="11" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>8</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="9"/>
-      <c r="D11" s="10"/>
+      <c r="D11" s="8"/>
       <c r="E11" s="2">
         <v>8</v>
       </c>
@@ -1485,13 +1485,13 @@
         <v>56</v>
       </c>
       <c r="K11" s="9"/>
-      <c r="L11" s="10"/>
+      <c r="L11" s="8"/>
       <c r="M11" s="2">
         <v>8</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
-      <c r="P11" s="8"/>
+      <c r="P11" s="10"/>
       <c r="Q11" s="5" t="b">
         <v>1</v>
       </c>
@@ -1508,9 +1508,9 @@
         <v>8</v>
       </c>
       <c r="X11" s="7"/>
-      <c r="AF11" s="8"/>
-    </row>
-    <row r="12" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF11" s="10"/>
+    </row>
+    <row r="12" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>9</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="9"/>
-      <c r="D12" s="10"/>
+      <c r="D12" s="8"/>
       <c r="E12" s="2">
         <v>9</v>
       </c>
@@ -1536,13 +1536,13 @@
         <v>57</v>
       </c>
       <c r="K12" s="9"/>
-      <c r="L12" s="10"/>
+      <c r="L12" s="8"/>
       <c r="M12" s="2">
         <v>9</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
-      <c r="P12" s="8"/>
+      <c r="P12" s="10"/>
       <c r="Q12" s="6" t="b">
         <v>0</v>
       </c>
@@ -1559,9 +1559,9 @@
         <v>9</v>
       </c>
       <c r="X12" s="7"/>
-      <c r="AF12" s="8"/>
-    </row>
-    <row r="13" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF12" s="10"/>
+    </row>
+    <row r="13" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>10</v>
       </c>
@@ -1571,7 +1571,7 @@
       <c r="C13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="10"/>
+      <c r="D13" s="8"/>
       <c r="E13" s="2">
         <v>10</v>
       </c>
@@ -1589,13 +1589,13 @@
       <c r="K13" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="L13" s="10"/>
+      <c r="L13" s="8"/>
       <c r="M13" s="2">
         <v>10</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
-      <c r="P13" s="8"/>
+      <c r="P13" s="10"/>
       <c r="Q13" s="6" t="b">
         <v>0</v>
       </c>
@@ -1612,9 +1612,9 @@
         <v>10</v>
       </c>
       <c r="X13" s="7"/>
-      <c r="AF13" s="8"/>
-    </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF13" s="10"/>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>11</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>12</v>
       </c>
       <c r="C14" s="9"/>
-      <c r="D14" s="10"/>
+      <c r="D14" s="8"/>
       <c r="E14" s="2">
         <v>11</v>
       </c>
@@ -1640,13 +1640,13 @@
         <v>59</v>
       </c>
       <c r="K14" s="9"/>
-      <c r="L14" s="10"/>
+      <c r="L14" s="8"/>
       <c r="M14" s="2">
         <v>11</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
-      <c r="P14" s="8"/>
+      <c r="P14" s="10"/>
       <c r="Q14" s="6" t="b">
         <v>0</v>
       </c>
@@ -1663,9 +1663,9 @@
         <v>11</v>
       </c>
       <c r="X14" s="7"/>
-      <c r="AF14" s="8"/>
-    </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF14" s="10"/>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>12</v>
       </c>
@@ -1675,7 +1675,7 @@
       <c r="C15" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="10"/>
+      <c r="D15" s="8"/>
       <c r="E15" s="2">
         <v>12</v>
       </c>
@@ -1687,13 +1687,13 @@
         <v>60</v>
       </c>
       <c r="K15" s="9"/>
-      <c r="L15" s="10"/>
+      <c r="L15" s="8"/>
       <c r="M15" s="2">
         <v>12</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
-      <c r="P15" s="8"/>
+      <c r="P15" s="10"/>
       <c r="Q15" s="6" t="b">
         <v>0</v>
       </c>
@@ -1710,9 +1710,9 @@
         <v>12</v>
       </c>
       <c r="X15" s="7"/>
-      <c r="AF15" s="8"/>
-    </row>
-    <row r="16" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF15" s="10"/>
+    </row>
+    <row r="16" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>13</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="9"/>
-      <c r="D16" s="10"/>
+      <c r="D16" s="8"/>
       <c r="E16" s="2">
         <v>13</v>
       </c>
@@ -1736,13 +1736,13 @@
       <c r="K16" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="L16" s="10"/>
+      <c r="L16" s="8"/>
       <c r="M16" s="2">
         <v>13</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
-      <c r="P16" s="8"/>
+      <c r="P16" s="10"/>
       <c r="Q16" s="6" t="b">
         <v>0</v>
       </c>
@@ -1759,9 +1759,9 @@
         <v>13</v>
       </c>
       <c r="X16" s="7"/>
-      <c r="AF16" s="8"/>
-    </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF16" s="10"/>
+    </row>
+    <row r="17" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>14</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="9"/>
-      <c r="D17" s="10"/>
+      <c r="D17" s="8"/>
       <c r="E17" s="2">
         <v>14</v>
       </c>
@@ -1787,13 +1787,13 @@
         <v>62</v>
       </c>
       <c r="K17" s="9"/>
-      <c r="L17" s="10"/>
+      <c r="L17" s="8"/>
       <c r="M17" s="2">
         <v>14</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
-      <c r="P17" s="8"/>
+      <c r="P17" s="10"/>
       <c r="Q17" s="6" t="b">
         <v>0</v>
       </c>
@@ -1810,9 +1810,9 @@
         <v>14</v>
       </c>
       <c r="X17" s="7"/>
-      <c r="AF17" s="8"/>
-    </row>
-    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF17" s="10"/>
+    </row>
+    <row r="18" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>15</v>
       </c>
@@ -1822,7 +1822,7 @@
       <c r="C18" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="10"/>
+      <c r="D18" s="8"/>
       <c r="E18" s="2">
         <v>15</v>
       </c>
@@ -1838,13 +1838,13 @@
         <v>63</v>
       </c>
       <c r="K18" s="9"/>
-      <c r="L18" s="10"/>
+      <c r="L18" s="8"/>
       <c r="M18" s="2">
         <v>15</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
-      <c r="P18" s="8"/>
+      <c r="P18" s="10"/>
       <c r="Q18" s="6" t="b">
         <v>0</v>
       </c>
@@ -1861,9 +1861,9 @@
         <v>15</v>
       </c>
       <c r="X18" s="7"/>
-      <c r="AF18" s="8"/>
-    </row>
-    <row r="19" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF18" s="10"/>
+    </row>
+    <row r="19" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>16</v>
       </c>
@@ -1871,7 +1871,7 @@
         <v>17</v>
       </c>
       <c r="C19" s="9"/>
-      <c r="D19" s="10"/>
+      <c r="D19" s="8"/>
       <c r="E19" s="2">
         <v>16</v>
       </c>
@@ -1889,13 +1889,13 @@
       <c r="K19" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="L19" s="10"/>
+      <c r="L19" s="8"/>
       <c r="M19" s="2">
         <v>16</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
-      <c r="P19" s="8"/>
+      <c r="P19" s="10"/>
       <c r="Q19" s="6" t="b">
         <v>0</v>
       </c>
@@ -1912,9 +1912,9 @@
         <v>16</v>
       </c>
       <c r="X19" s="7"/>
-      <c r="AF19" s="8"/>
-    </row>
-    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF19" s="10"/>
+    </row>
+    <row r="20" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>17</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>18</v>
       </c>
       <c r="C20" s="9"/>
-      <c r="D20" s="10"/>
+      <c r="D20" s="8"/>
       <c r="E20" s="2">
         <v>17</v>
       </c>
@@ -1940,17 +1940,17 @@
         <v>65</v>
       </c>
       <c r="K20" s="9"/>
-      <c r="L20" s="10"/>
+      <c r="L20" s="8"/>
       <c r="M20" s="2">
         <v>17</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
-      <c r="P20" s="8"/>
+      <c r="P20" s="10"/>
       <c r="X20" s="7"/>
-      <c r="AF20" s="8"/>
-    </row>
-    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF20" s="10"/>
+    </row>
+    <row r="21" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>18</v>
       </c>
@@ -1960,7 +1960,7 @@
       <c r="C21" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D21" s="10"/>
+      <c r="D21" s="8"/>
       <c r="E21" s="2">
         <v>18</v>
       </c>
@@ -1976,17 +1976,17 @@
         <v>66</v>
       </c>
       <c r="K21" s="9"/>
-      <c r="L21" s="10"/>
+      <c r="L21" s="8"/>
       <c r="M21" s="2">
         <v>18</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
-      <c r="P21" s="8"/>
+      <c r="P21" s="10"/>
       <c r="X21" s="7"/>
-      <c r="AF21" s="8"/>
-    </row>
-    <row r="22" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF21" s="10"/>
+    </row>
+    <row r="22" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>19</v>
       </c>
@@ -1994,7 +1994,7 @@
         <v>28</v>
       </c>
       <c r="C22" s="9"/>
-      <c r="D22" s="10"/>
+      <c r="D22" s="8"/>
       <c r="E22" s="2">
         <v>19</v>
       </c>
@@ -2012,17 +2012,17 @@
       <c r="K22" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="L22" s="10"/>
+      <c r="L22" s="8"/>
       <c r="M22" s="2">
         <v>19</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
-      <c r="P22" s="8"/>
+      <c r="P22" s="10"/>
       <c r="X22" s="7"/>
-      <c r="AF22" s="8"/>
-    </row>
-    <row r="23" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF22" s="10"/>
+    </row>
+    <row r="23" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>20</v>
       </c>
@@ -2030,7 +2030,7 @@
         <v>29</v>
       </c>
       <c r="C23" s="9"/>
-      <c r="D23" s="10"/>
+      <c r="D23" s="8"/>
       <c r="E23" s="2">
         <v>20</v>
       </c>
@@ -2048,17 +2048,17 @@
         <v>70</v>
       </c>
       <c r="K23" s="9"/>
-      <c r="L23" s="10"/>
+      <c r="L23" s="8"/>
       <c r="M23" s="2">
         <v>20</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
-      <c r="P23" s="8"/>
+      <c r="P23" s="10"/>
       <c r="X23" s="7"/>
-      <c r="AF23" s="8"/>
-    </row>
-    <row r="24" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF23" s="10"/>
+    </row>
+    <row r="24" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>21</v>
       </c>
@@ -2068,7 +2068,7 @@
       <c r="C24" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="10"/>
+      <c r="D24" s="8"/>
       <c r="E24" s="2">
         <v>21</v>
       </c>
@@ -2084,17 +2084,17 @@
         <v>71</v>
       </c>
       <c r="K24" s="9"/>
-      <c r="L24" s="10"/>
+      <c r="L24" s="8"/>
       <c r="M24" s="2">
         <v>21</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
-      <c r="P24" s="8"/>
+      <c r="P24" s="10"/>
       <c r="X24" s="7"/>
-      <c r="AF24" s="8"/>
-    </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF24" s="10"/>
+    </row>
+    <row r="25" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>22</v>
       </c>
@@ -2102,7 +2102,7 @@
         <v>34</v>
       </c>
       <c r="C25" s="9"/>
-      <c r="D25" s="10"/>
+      <c r="D25" s="8"/>
       <c r="E25" s="2">
         <v>22</v>
       </c>
@@ -2118,17 +2118,17 @@
         <v>88</v>
       </c>
       <c r="K25" s="9"/>
-      <c r="L25" s="10"/>
+      <c r="L25" s="8"/>
       <c r="M25" s="2">
         <v>22</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
-      <c r="P25" s="8"/>
+      <c r="P25" s="10"/>
       <c r="X25" s="7"/>
-      <c r="AF25" s="8"/>
-    </row>
-    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF25" s="10"/>
+    </row>
+    <row r="26" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>23</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>35</v>
       </c>
       <c r="C26" s="9"/>
-      <c r="D26" s="10"/>
+      <c r="D26" s="8"/>
       <c r="E26" s="2">
         <v>23</v>
       </c>
@@ -2156,17 +2156,17 @@
       <c r="K26" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="L26" s="10"/>
+      <c r="L26" s="8"/>
       <c r="M26" s="2">
         <v>23</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
-      <c r="P26" s="8"/>
+      <c r="P26" s="10"/>
       <c r="X26" s="7"/>
-      <c r="AF26" s="8"/>
-    </row>
-    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF26" s="10"/>
+    </row>
+    <row r="27" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>24</v>
       </c>
@@ -2176,7 +2176,7 @@
       <c r="C27" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="10"/>
+      <c r="D27" s="8"/>
       <c r="E27" s="2">
         <v>24</v>
       </c>
@@ -2192,17 +2192,17 @@
         <v>84</v>
       </c>
       <c r="K27" s="9"/>
-      <c r="L27" s="10"/>
+      <c r="L27" s="8"/>
       <c r="M27" s="2">
         <v>24</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
-      <c r="P27" s="8"/>
+      <c r="P27" s="10"/>
       <c r="X27" s="7"/>
-      <c r="AF27" s="8"/>
-    </row>
-    <row r="28" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF27" s="10"/>
+    </row>
+    <row r="28" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>25</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>31</v>
       </c>
       <c r="C28" s="9"/>
-      <c r="D28" s="10"/>
+      <c r="D28" s="8"/>
       <c r="E28" s="2">
         <v>25</v>
       </c>
@@ -2226,17 +2226,17 @@
         <v>85</v>
       </c>
       <c r="K28" s="9"/>
-      <c r="L28" s="10"/>
+      <c r="L28" s="8"/>
       <c r="M28" s="2">
         <v>25</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
-      <c r="P28" s="8"/>
+      <c r="P28" s="10"/>
       <c r="X28" s="7"/>
-      <c r="AF28" s="8"/>
-    </row>
-    <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF28" s="10"/>
+    </row>
+    <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>26</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>32</v>
       </c>
       <c r="C29" s="9"/>
-      <c r="D29" s="10"/>
+      <c r="D29" s="8"/>
       <c r="E29" s="2">
         <v>26</v>
       </c>
@@ -2262,17 +2262,17 @@
         <v>109</v>
       </c>
       <c r="K29" s="2"/>
-      <c r="L29" s="10"/>
+      <c r="L29" s="8"/>
       <c r="M29" s="2">
         <v>26</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
-      <c r="P29" s="8"/>
+      <c r="P29" s="10"/>
       <c r="X29" s="7"/>
-      <c r="AF29" s="8"/>
-    </row>
-    <row r="30" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF29" s="10"/>
+    </row>
+    <row r="30" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>27</v>
       </c>
@@ -2282,7 +2282,7 @@
       <c r="C30" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D30" s="10"/>
+      <c r="D30" s="8"/>
       <c r="E30" s="2">
         <v>27</v>
       </c>
@@ -2298,17 +2298,17 @@
         <v>90</v>
       </c>
       <c r="K30" s="2"/>
-      <c r="L30" s="10"/>
+      <c r="L30" s="8"/>
       <c r="M30" s="2">
         <v>27</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
-      <c r="P30" s="8"/>
+      <c r="P30" s="10"/>
       <c r="X30" s="7"/>
-      <c r="AF30" s="8"/>
-    </row>
-    <row r="31" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF30" s="10"/>
+    </row>
+    <row r="31" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>28</v>
       </c>
@@ -2316,7 +2316,7 @@
         <v>38</v>
       </c>
       <c r="C31" s="9"/>
-      <c r="D31" s="10"/>
+      <c r="D31" s="8"/>
       <c r="E31" s="2">
         <v>28</v>
       </c>
@@ -2332,17 +2332,17 @@
         <v>103</v>
       </c>
       <c r="K31" s="2"/>
-      <c r="L31" s="10"/>
+      <c r="L31" s="8"/>
       <c r="M31" s="2">
         <v>28</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
-      <c r="P31" s="8"/>
+      <c r="P31" s="10"/>
       <c r="X31" s="7"/>
-      <c r="AF31" s="8"/>
-    </row>
-    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF31" s="10"/>
+    </row>
+    <row r="32" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>29</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>39</v>
       </c>
       <c r="C32" s="9"/>
-      <c r="D32" s="10"/>
+      <c r="D32" s="8"/>
       <c r="E32" s="2">
         <v>29</v>
       </c>
@@ -2368,17 +2368,17 @@
       <c r="K32" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="L32" s="10"/>
+      <c r="L32" s="8"/>
       <c r="M32" s="2">
         <v>29</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
-      <c r="P32" s="8"/>
+      <c r="P32" s="10"/>
       <c r="X32" s="7"/>
-      <c r="AF32" s="8"/>
-    </row>
-    <row r="33" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF32" s="10"/>
+    </row>
+    <row r="33" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>30</v>
       </c>
@@ -2388,7 +2388,7 @@
       <c r="C33" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D33" s="10"/>
+      <c r="D33" s="8"/>
       <c r="E33" s="2">
         <v>30</v>
       </c>
@@ -2406,17 +2406,17 @@
         <v>110</v>
       </c>
       <c r="K33" s="2"/>
-      <c r="L33" s="10"/>
+      <c r="L33" s="8"/>
       <c r="M33" s="2">
         <v>30</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
-      <c r="P33" s="8"/>
+      <c r="P33" s="10"/>
       <c r="X33" s="7"/>
-      <c r="AF33" s="8"/>
-    </row>
-    <row r="34" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF33" s="10"/>
+    </row>
+    <row r="34" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>31</v>
       </c>
@@ -2426,7 +2426,7 @@
       <c r="C34" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D34" s="10"/>
+      <c r="D34" s="8"/>
       <c r="E34" s="2">
         <v>31</v>
       </c>
@@ -2442,17 +2442,17 @@
         <v>120</v>
       </c>
       <c r="K34" s="2"/>
-      <c r="L34" s="10"/>
+      <c r="L34" s="8"/>
       <c r="M34" s="2">
         <v>31</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
-      <c r="P34" s="8"/>
+      <c r="P34" s="10"/>
       <c r="X34" s="7"/>
-      <c r="AF34" s="8"/>
-    </row>
-    <row r="35" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF34" s="10"/>
+    </row>
+    <row r="35" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>32</v>
       </c>
@@ -2460,7 +2460,7 @@
         <v>53</v>
       </c>
       <c r="C35" s="9"/>
-      <c r="D35" s="10"/>
+      <c r="D35" s="8"/>
       <c r="E35" s="2">
         <v>32</v>
       </c>
@@ -2474,17 +2474,17 @@
       </c>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
-      <c r="L35" s="10"/>
+      <c r="L35" s="8"/>
       <c r="M35" s="2">
         <v>32</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
-      <c r="P35" s="8"/>
+      <c r="P35" s="10"/>
       <c r="X35" s="7"/>
-      <c r="AF35" s="8"/>
-    </row>
-    <row r="36" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF35" s="10"/>
+    </row>
+    <row r="36" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A36" s="11"/>
       <c r="B36" s="12"/>
       <c r="C36" s="12"/>
@@ -2501,53 +2501,53 @@
       <c r="N36" s="12"/>
       <c r="O36" s="13"/>
     </row>
-    <row r="37" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
       <c r="H37" s="14"/>
-      <c r="I37" s="10" t="s">
+      <c r="I37" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="J37" s="10"/>
-      <c r="K37" s="10"/>
-      <c r="L37" s="10"/>
-      <c r="M37" s="10"/>
-      <c r="N37" s="10"/>
-      <c r="O37" s="10"/>
-    </row>
-    <row r="38" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8"/>
+      <c r="N37" s="8"/>
+      <c r="O37" s="8"/>
+    </row>
+    <row r="38" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A38" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10" t="s">
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="F38" s="10"/>
-      <c r="G38" s="10"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
       <c r="H38" s="15"/>
-      <c r="I38" s="10" t="s">
+      <c r="I38" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="J38" s="10"/>
-      <c r="K38" s="10"/>
-      <c r="L38" s="10"/>
-      <c r="M38" s="10" t="s">
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="N38" s="10"/>
-      <c r="O38" s="10"/>
-    </row>
-    <row r="39" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="N38" s="8"/>
+      <c r="O38" s="8"/>
+    </row>
+    <row r="39" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>0</v>
       </c>
@@ -2557,7 +2557,7 @@
       <c r="C39" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D39" s="10"/>
+      <c r="D39" s="8"/>
       <c r="E39" s="3" t="s">
         <v>0</v>
       </c>
@@ -2577,7 +2577,7 @@
       <c r="K39" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="L39" s="10"/>
+      <c r="L39" s="8"/>
       <c r="M39" s="3" t="s">
         <v>0</v>
       </c>
@@ -2588,7 +2588,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>1</v>
       </c>
@@ -2598,7 +2598,7 @@
       <c r="C40" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D40" s="10"/>
+      <c r="D40" s="8"/>
       <c r="E40" s="2">
         <v>1</v>
       </c>
@@ -2614,14 +2614,14 @@
       <c r="K40" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="L40" s="10"/>
+      <c r="L40" s="8"/>
       <c r="M40" s="2">
         <v>1</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
     </row>
-    <row r="41" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>2</v>
       </c>
@@ -2629,7 +2629,7 @@
         <v>3</v>
       </c>
       <c r="C41" s="9"/>
-      <c r="D41" s="10"/>
+      <c r="D41" s="8"/>
       <c r="E41" s="2">
         <v>2</v>
       </c>
@@ -2643,14 +2643,14 @@
         <v>3</v>
       </c>
       <c r="K41" s="9"/>
-      <c r="L41" s="10"/>
+      <c r="L41" s="8"/>
       <c r="M41" s="2">
         <v>2</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
     </row>
-    <row r="42" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>3</v>
       </c>
@@ -2658,7 +2658,7 @@
         <v>4</v>
       </c>
       <c r="C42" s="9"/>
-      <c r="D42" s="10"/>
+      <c r="D42" s="8"/>
       <c r="E42" s="2">
         <v>3</v>
       </c>
@@ -2672,14 +2672,14 @@
         <v>4</v>
       </c>
       <c r="K42" s="9"/>
-      <c r="L42" s="10"/>
+      <c r="L42" s="8"/>
       <c r="M42" s="2">
         <v>3</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
     </row>
-    <row r="43" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>4</v>
       </c>
@@ -2689,7 +2689,7 @@
       <c r="C43" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D43" s="10"/>
+      <c r="D43" s="8"/>
       <c r="E43" s="2">
         <v>4</v>
       </c>
@@ -2703,14 +2703,14 @@
         <v>5</v>
       </c>
       <c r="K43" s="9"/>
-      <c r="L43" s="10"/>
+      <c r="L43" s="8"/>
       <c r="M43" s="2">
         <v>4</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
     </row>
-    <row r="44" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>5</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>6</v>
       </c>
       <c r="C44" s="9"/>
-      <c r="D44" s="10"/>
+      <c r="D44" s="8"/>
       <c r="E44" s="2">
         <v>5</v>
       </c>
@@ -2732,14 +2732,14 @@
         <v>6</v>
       </c>
       <c r="K44" s="9"/>
-      <c r="L44" s="10"/>
+      <c r="L44" s="8"/>
       <c r="M44" s="2">
         <v>5</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
     </row>
-    <row r="45" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>6</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>7</v>
       </c>
       <c r="C45" s="9"/>
-      <c r="D45" s="10"/>
+      <c r="D45" s="8"/>
       <c r="E45" s="2">
         <v>6</v>
       </c>
@@ -2761,14 +2761,14 @@
         <v>7</v>
       </c>
       <c r="K45" s="9"/>
-      <c r="L45" s="10"/>
+      <c r="L45" s="8"/>
       <c r="M45" s="2">
         <v>6</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
     </row>
-    <row r="46" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>7</v>
       </c>
@@ -2778,7 +2778,7 @@
       <c r="C46" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D46" s="10"/>
+      <c r="D46" s="8"/>
       <c r="E46" s="2">
         <v>7</v>
       </c>
@@ -2792,14 +2792,14 @@
         <v>91</v>
       </c>
       <c r="K46" s="9"/>
-      <c r="L46" s="10"/>
+      <c r="L46" s="8"/>
       <c r="M46" s="2">
         <v>7</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
     </row>
-    <row r="47" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>8</v>
       </c>
@@ -2807,7 +2807,7 @@
         <v>56</v>
       </c>
       <c r="C47" s="9"/>
-      <c r="D47" s="10"/>
+      <c r="D47" s="8"/>
       <c r="E47" s="2">
         <v>8</v>
       </c>
@@ -2821,14 +2821,14 @@
         <v>92</v>
       </c>
       <c r="K47" s="9"/>
-      <c r="L47" s="10"/>
+      <c r="L47" s="8"/>
       <c r="M47" s="2">
         <v>8</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
     </row>
-    <row r="48" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>9</v>
       </c>
@@ -2836,7 +2836,7 @@
         <v>57</v>
       </c>
       <c r="C48" s="9"/>
-      <c r="D48" s="10"/>
+      <c r="D48" s="8"/>
       <c r="E48" s="2">
         <v>9</v>
       </c>
@@ -2850,14 +2850,14 @@
         <v>93</v>
       </c>
       <c r="K48" s="9"/>
-      <c r="L48" s="10"/>
+      <c r="L48" s="8"/>
       <c r="M48" s="2">
         <v>9</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>10</v>
       </c>
@@ -2867,7 +2867,7 @@
       <c r="C49" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="D49" s="10"/>
+      <c r="D49" s="8"/>
       <c r="E49" s="2">
         <v>10</v>
       </c>
@@ -2881,14 +2881,14 @@
         <v>94</v>
       </c>
       <c r="K49" s="9"/>
-      <c r="L49" s="10"/>
+      <c r="L49" s="8"/>
       <c r="M49" s="2">
         <v>10</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>11</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>59</v>
       </c>
       <c r="C50" s="9"/>
-      <c r="D50" s="10"/>
+      <c r="D50" s="8"/>
       <c r="E50" s="2">
         <v>11</v>
       </c>
@@ -2910,14 +2910,14 @@
         <v>95</v>
       </c>
       <c r="K50" s="9"/>
-      <c r="L50" s="10"/>
+      <c r="L50" s="8"/>
       <c r="M50" s="2">
         <v>11</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>12</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>60</v>
       </c>
       <c r="C51" s="9"/>
-      <c r="D51" s="10"/>
+      <c r="D51" s="8"/>
       <c r="E51" s="2">
         <v>12</v>
       </c>
@@ -2939,14 +2939,14 @@
         <v>96</v>
       </c>
       <c r="K51" s="9"/>
-      <c r="L51" s="10"/>
+      <c r="L51" s="8"/>
       <c r="M51" s="2">
         <v>12</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>13</v>
       </c>
@@ -2956,7 +2956,7 @@
       <c r="C52" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="D52" s="10"/>
+      <c r="D52" s="8"/>
       <c r="E52" s="2">
         <v>13</v>
       </c>
@@ -2972,14 +2972,14 @@
       <c r="K52" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="L52" s="10"/>
+      <c r="L52" s="8"/>
       <c r="M52" s="2">
         <v>13</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>14</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>62</v>
       </c>
       <c r="C53" s="9"/>
-      <c r="D53" s="10"/>
+      <c r="D53" s="8"/>
       <c r="E53" s="2">
         <v>14</v>
       </c>
@@ -3001,14 +3001,14 @@
         <v>98</v>
       </c>
       <c r="K53" s="9"/>
-      <c r="L53" s="10"/>
+      <c r="L53" s="8"/>
       <c r="M53" s="2">
         <v>14</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>15</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>63</v>
       </c>
       <c r="C54" s="9"/>
-      <c r="D54" s="10"/>
+      <c r="D54" s="8"/>
       <c r="E54" s="2">
         <v>15</v>
       </c>
@@ -3030,14 +3030,14 @@
         <v>99</v>
       </c>
       <c r="K54" s="9"/>
-      <c r="L54" s="10"/>
+      <c r="L54" s="8"/>
       <c r="M54" s="2">
         <v>15</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>16</v>
       </c>
@@ -3047,7 +3047,7 @@
       <c r="C55" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="D55" s="10"/>
+      <c r="D55" s="8"/>
       <c r="E55" s="2">
         <v>16</v>
       </c>
@@ -3063,14 +3063,14 @@
       <c r="K55" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="L55" s="10"/>
+      <c r="L55" s="8"/>
       <c r="M55" s="2">
         <v>16</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>17</v>
       </c>
@@ -3078,7 +3078,7 @@
         <v>65</v>
       </c>
       <c r="C56" s="9"/>
-      <c r="D56" s="10"/>
+      <c r="D56" s="8"/>
       <c r="E56" s="2">
         <v>17</v>
       </c>
@@ -3092,14 +3092,14 @@
         <v>103</v>
       </c>
       <c r="K56" s="4"/>
-      <c r="L56" s="10"/>
+      <c r="L56" s="8"/>
       <c r="M56" s="2">
         <v>17</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>18</v>
       </c>
@@ -3107,7 +3107,7 @@
         <v>66</v>
       </c>
       <c r="C57" s="9"/>
-      <c r="D57" s="10"/>
+      <c r="D57" s="8"/>
       <c r="E57" s="2">
         <v>18</v>
       </c>
@@ -3121,14 +3121,14 @@
         <v>109</v>
       </c>
       <c r="K57" s="4"/>
-      <c r="L57" s="10"/>
+      <c r="L57" s="8"/>
       <c r="M57" s="2">
         <v>18</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
     </row>
-    <row r="58" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>19</v>
       </c>
@@ -3138,7 +3138,7 @@
       <c r="C58" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D58" s="10"/>
+      <c r="D58" s="8"/>
       <c r="E58" s="2">
         <v>19</v>
       </c>
@@ -3154,14 +3154,14 @@
       <c r="K58" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="L58" s="10"/>
+      <c r="L58" s="8"/>
       <c r="M58" s="2">
         <v>19</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>20</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>70</v>
       </c>
       <c r="C59" s="9"/>
-      <c r="D59" s="10"/>
+      <c r="D59" s="8"/>
       <c r="E59" s="2">
         <v>20</v>
       </c>
@@ -3183,14 +3183,14 @@
         <v>107</v>
       </c>
       <c r="K59" s="4"/>
-      <c r="L59" s="10"/>
+      <c r="L59" s="8"/>
       <c r="M59" s="2">
         <v>20</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>21</v>
       </c>
@@ -3198,7 +3198,7 @@
         <v>71</v>
       </c>
       <c r="C60" s="9"/>
-      <c r="D60" s="10"/>
+      <c r="D60" s="8"/>
       <c r="E60" s="2">
         <v>21</v>
       </c>
@@ -3210,14 +3210,14 @@
       </c>
       <c r="J60" s="2"/>
       <c r="K60" s="4"/>
-      <c r="L60" s="10"/>
+      <c r="L60" s="8"/>
       <c r="M60" s="2">
         <v>21</v>
       </c>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>22</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>88</v>
       </c>
       <c r="C61" s="9"/>
-      <c r="D61" s="10"/>
+      <c r="D61" s="8"/>
       <c r="E61" s="2">
         <v>22</v>
       </c>
@@ -3237,14 +3237,14 @@
       </c>
       <c r="J61" s="2"/>
       <c r="K61" s="4"/>
-      <c r="L61" s="10"/>
+      <c r="L61" s="8"/>
       <c r="M61" s="2">
         <v>22</v>
       </c>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
     </row>
-    <row r="62" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>23</v>
       </c>
@@ -3254,7 +3254,7 @@
       <c r="C62" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D62" s="10"/>
+      <c r="D62" s="8"/>
       <c r="E62" s="2">
         <v>23</v>
       </c>
@@ -3266,14 +3266,14 @@
       </c>
       <c r="J62" s="2"/>
       <c r="K62" s="4"/>
-      <c r="L62" s="10"/>
+      <c r="L62" s="8"/>
       <c r="M62" s="2">
         <v>23</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>24</v>
       </c>
@@ -3281,7 +3281,7 @@
         <v>84</v>
       </c>
       <c r="C63" s="2"/>
-      <c r="D63" s="10"/>
+      <c r="D63" s="8"/>
       <c r="E63" s="2">
         <v>24</v>
       </c>
@@ -3293,14 +3293,14 @@
       </c>
       <c r="J63" s="2"/>
       <c r="K63" s="4"/>
-      <c r="L63" s="10"/>
+      <c r="L63" s="8"/>
       <c r="M63" s="2">
         <v>24</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>25</v>
       </c>
@@ -3308,7 +3308,7 @@
         <v>85</v>
       </c>
       <c r="C64" s="2"/>
-      <c r="D64" s="10"/>
+      <c r="D64" s="8"/>
       <c r="E64" s="2">
         <v>25</v>
       </c>
@@ -3320,14 +3320,14 @@
       </c>
       <c r="J64" s="2"/>
       <c r="K64" s="4"/>
-      <c r="L64" s="10"/>
+      <c r="L64" s="8"/>
       <c r="M64" s="2">
         <v>25</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>26</v>
       </c>
@@ -3337,7 +3337,7 @@
       <c r="C65" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D65" s="10"/>
+      <c r="D65" s="8"/>
       <c r="E65" s="2">
         <v>26</v>
       </c>
@@ -3349,14 +3349,14 @@
       </c>
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
-      <c r="L65" s="10"/>
+      <c r="L65" s="8"/>
       <c r="M65" s="2">
         <v>26</v>
       </c>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>27</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>120</v>
       </c>
       <c r="C66" s="2"/>
-      <c r="D66" s="10"/>
+      <c r="D66" s="8"/>
       <c r="E66" s="2">
         <v>27</v>
       </c>
@@ -3376,20 +3376,20 @@
       </c>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
-      <c r="L66" s="10"/>
+      <c r="L66" s="8"/>
       <c r="M66" s="2">
         <v>27</v>
       </c>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>28</v>
       </c>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
-      <c r="D67" s="10"/>
+      <c r="D67" s="8"/>
       <c r="E67" s="2">
         <v>28</v>
       </c>
@@ -3401,20 +3401,20 @@
       </c>
       <c r="J67" s="2"/>
       <c r="K67" s="2"/>
-      <c r="L67" s="10"/>
+      <c r="L67" s="8"/>
       <c r="M67" s="2">
         <v>28</v>
       </c>
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>29</v>
       </c>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
-      <c r="D68" s="10"/>
+      <c r="D68" s="8"/>
       <c r="E68" s="2">
         <v>29</v>
       </c>
@@ -3426,20 +3426,20 @@
       </c>
       <c r="J68" s="2"/>
       <c r="K68" s="2"/>
-      <c r="L68" s="10"/>
+      <c r="L68" s="8"/>
       <c r="M68" s="2">
         <v>29</v>
       </c>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>30</v>
       </c>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
-      <c r="D69" s="10"/>
+      <c r="D69" s="8"/>
       <c r="E69" s="2">
         <v>30</v>
       </c>
@@ -3451,20 +3451,20 @@
       </c>
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
-      <c r="L69" s="10"/>
+      <c r="L69" s="8"/>
       <c r="M69" s="2">
         <v>30</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>31</v>
       </c>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
-      <c r="D70" s="10"/>
+      <c r="D70" s="8"/>
       <c r="E70" s="2">
         <v>31</v>
       </c>
@@ -3476,20 +3476,20 @@
       </c>
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
-      <c r="L70" s="10"/>
+      <c r="L70" s="8"/>
       <c r="M70" s="2">
         <v>31</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>32</v>
       </c>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
-      <c r="D71" s="10"/>
+      <c r="D71" s="8"/>
       <c r="E71" s="2">
         <v>32</v>
       </c>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="J71" s="2"/>
       <c r="K71" s="2"/>
-      <c r="L71" s="10"/>
+      <c r="L71" s="8"/>
       <c r="M71" s="2">
         <v>32</v>
       </c>
@@ -3510,6 +3510,50 @@
     </row>
   </sheetData>
   <mergeCells count="60">
+    <mergeCell ref="Q1:U1"/>
+    <mergeCell ref="C52:C54"/>
+    <mergeCell ref="G20:G22"/>
+    <mergeCell ref="G23:G25"/>
+    <mergeCell ref="G26:G28"/>
+    <mergeCell ref="I1:O1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:L35"/>
+    <mergeCell ref="M2:O2"/>
+    <mergeCell ref="K4:K6"/>
+    <mergeCell ref="K7:K9"/>
+    <mergeCell ref="K10:K12"/>
+    <mergeCell ref="K13:K15"/>
+    <mergeCell ref="K16:K18"/>
+    <mergeCell ref="K19:K21"/>
+    <mergeCell ref="K22:K25"/>
+    <mergeCell ref="K26:K28"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:D71"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="D2:D35"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="G17:G19"/>
+    <mergeCell ref="G33:G35"/>
+    <mergeCell ref="G29:G32"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="C27:C29"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="C21:C23"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="C15:C17"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="G4:G5"/>
@@ -3526,50 +3570,6 @@
     <mergeCell ref="H1:H35"/>
     <mergeCell ref="C10:C12"/>
     <mergeCell ref="C7:C9"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="C27:C29"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="C21:C23"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="C15:C17"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="G17:G19"/>
-    <mergeCell ref="G33:G35"/>
-    <mergeCell ref="G29:G32"/>
-    <mergeCell ref="K26:K28"/>
-    <mergeCell ref="A37:G37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:D71"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="C55:C57"/>
-    <mergeCell ref="D2:D35"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="C30:C32"/>
-    <mergeCell ref="Q1:U1"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="G20:G22"/>
-    <mergeCell ref="G23:G25"/>
-    <mergeCell ref="G26:G28"/>
-    <mergeCell ref="I1:O1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:L35"/>
-    <mergeCell ref="M2:O2"/>
-    <mergeCell ref="K4:K6"/>
-    <mergeCell ref="K7:K9"/>
-    <mergeCell ref="K10:K12"/>
-    <mergeCell ref="K13:K15"/>
-    <mergeCell ref="K16:K18"/>
-    <mergeCell ref="K19:K21"/>
-    <mergeCell ref="K22:K25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
only EVA left now
</commit_message>
<xml_diff>
--- a/documentation/parts and their channels.xlsx
+++ b/documentation/parts and their channels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Squingle\Desktop\!folders\! d-github\EISS\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB78BD11-35A0-45E7-B9D1-66BA854F8990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B0C664-EEA1-4629-8040-D1414B9D1799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="3600" windowWidth="29040" windowHeight="15720" xr2:uid="{A0965BB0-A002-463F-9819-73939F3991DC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A0965BB0-A002-463F-9819-73939F3991DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="123">
   <si>
     <t>Freq:</t>
   </si>
@@ -393,6 +393,18 @@
   </si>
   <si>
     <t>friendly selected</t>
+  </si>
+  <si>
+    <t>friend selected1 x</t>
+  </si>
+  <si>
+    <t>friend selected1 y</t>
+  </si>
+  <si>
+    <t>friend selected1 z</t>
+  </si>
+  <si>
+    <t>friendly selected transmit 1</t>
   </si>
 </sst>
 </file>
@@ -576,13 +588,28 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -605,21 +632,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -973,60 +985,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="9" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7" t="s">
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
-      <c r="T1" s="7"/>
-      <c r="U1" s="7"/>
-      <c r="AF1" s="7"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="AF1" s="14"/>
     </row>
     <row r="2" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9" t="s">
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="9" t="s">
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9" t="s">
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="N2" s="9"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="7"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="14"/>
       <c r="Q2" s="1" t="s">
         <v>88</v>
       </c>
@@ -1039,7 +1051,7 @@
       <c r="T2" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="AF2" s="7"/>
+      <c r="AF2" s="14"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -1051,7 +1063,7 @@
       <c r="C3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="9"/>
+      <c r="D3" s="10"/>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1061,7 +1073,7 @@
       <c r="G3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="16"/>
+      <c r="H3" s="21"/>
       <c r="I3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1071,7 +1083,7 @@
       <c r="K3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="9"/>
+      <c r="L3" s="10"/>
       <c r="M3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1081,7 +1093,7 @@
       <c r="O3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="P3" s="7"/>
+      <c r="P3" s="14"/>
       <c r="Q3" s="1" t="s">
         <v>89</v>
       </c>
@@ -1097,7 +1109,7 @@
       <c r="U3" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="AF3" s="7"/>
+      <c r="AF3" s="14"/>
     </row>
     <row r="4" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -1106,36 +1118,36 @@
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="9"/>
+      <c r="D4" s="10"/>
       <c r="E4" s="2">
         <v>1</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="16"/>
+      <c r="H4" s="21"/>
       <c r="I4" s="2">
         <v>1</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="9"/>
+      <c r="L4" s="10"/>
       <c r="M4" s="2">
         <v>1</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
-      <c r="P4" s="7"/>
+      <c r="P4" s="14"/>
       <c r="Q4" s="5" t="b">
         <v>1</v>
       </c>
@@ -1151,7 +1163,7 @@
       <c r="U4" s="1">
         <v>1</v>
       </c>
-      <c r="AF4" s="7"/>
+      <c r="AF4" s="14"/>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -1160,30 +1172,30 @@
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="10"/>
       <c r="E5" s="2">
         <v>2</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="8"/>
-      <c r="H5" s="16"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="21"/>
       <c r="I5" s="2">
         <v>2</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K5" s="8"/>
-      <c r="L5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="10"/>
       <c r="M5" s="2">
         <v>2</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
-      <c r="P5" s="7"/>
+      <c r="P5" s="14"/>
       <c r="Q5" s="5" t="b">
         <v>1</v>
       </c>
@@ -1199,7 +1211,7 @@
       <c r="U5" s="1">
         <v>2</v>
       </c>
-      <c r="AF5" s="7"/>
+      <c r="AF5" s="14"/>
     </row>
     <row r="6" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -1208,8 +1220,8 @@
       <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="10"/>
       <c r="E6" s="2">
         <v>3</v>
       </c>
@@ -1219,21 +1231,21 @@
       <c r="G6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H6" s="16"/>
+      <c r="H6" s="21"/>
       <c r="I6" s="2">
         <v>3</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K6" s="8"/>
-      <c r="L6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="10"/>
       <c r="M6" s="2">
         <v>3</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
-      <c r="P6" s="7"/>
+      <c r="P6" s="14"/>
       <c r="Q6" s="5" t="b">
         <v>1</v>
       </c>
@@ -1249,7 +1261,7 @@
       <c r="U6" s="1">
         <v>3</v>
       </c>
-      <c r="AF6" s="7"/>
+      <c r="AF6" s="14"/>
     </row>
     <row r="7" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -1258,32 +1270,32 @@
       <c r="B7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="9"/>
+      <c r="D7" s="10"/>
       <c r="E7" s="2">
         <v>4</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="16"/>
+      <c r="H7" s="21"/>
       <c r="I7" s="2">
         <v>4</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="K7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="9"/>
+      <c r="L7" s="10"/>
       <c r="M7" s="2">
         <v>4</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
-      <c r="P7" s="7"/>
+      <c r="P7" s="14"/>
       <c r="Q7" s="5" t="b">
         <v>1</v>
       </c>
@@ -1299,7 +1311,7 @@
       <c r="U7" s="1">
         <v>4</v>
       </c>
-      <c r="AF7" s="7"/>
+      <c r="AF7" s="14"/>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -1308,28 +1320,28 @@
       <c r="B8" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="10"/>
       <c r="E8" s="2">
         <v>5</v>
       </c>
       <c r="F8" s="2"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="16"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="21"/>
       <c r="I8" s="2">
         <v>5</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="K8" s="8"/>
-      <c r="L8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="10"/>
       <c r="M8" s="2">
         <v>5</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
-      <c r="P8" s="7"/>
+      <c r="P8" s="14"/>
       <c r="Q8" s="5" t="b">
         <v>1</v>
       </c>
@@ -1345,7 +1357,7 @@
       <c r="U8" s="1">
         <v>5</v>
       </c>
-      <c r="AF8" s="7"/>
+      <c r="AF8" s="14"/>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -1354,28 +1366,28 @@
       <c r="B9" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="10"/>
       <c r="E9" s="2">
         <v>6</v>
       </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="16"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="21"/>
       <c r="I9" s="2">
         <v>6</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="K9" s="8"/>
-      <c r="L9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="10"/>
       <c r="M9" s="2">
         <v>6</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-      <c r="P9" s="7"/>
+      <c r="P9" s="14"/>
       <c r="Q9" s="5" t="b">
         <v>1</v>
       </c>
@@ -1391,7 +1403,7 @@
       <c r="U9" s="1">
         <v>6</v>
       </c>
-      <c r="AF9" s="7"/>
+      <c r="AF9" s="14"/>
     </row>
     <row r="10" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -1400,36 +1412,36 @@
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="9"/>
+      <c r="D10" s="10"/>
       <c r="E10" s="2">
         <v>7</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="16"/>
+      <c r="H10" s="21"/>
       <c r="I10" s="2">
         <v>7</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="K10" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="L10" s="9"/>
+      <c r="L10" s="10"/>
       <c r="M10" s="2">
         <v>7</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-      <c r="P10" s="7"/>
+      <c r="P10" s="14"/>
       <c r="Q10" s="5" t="b">
         <v>1</v>
       </c>
@@ -1445,7 +1457,7 @@
       <c r="U10" s="1">
         <v>7</v>
       </c>
-      <c r="AF10" s="7"/>
+      <c r="AF10" s="14"/>
     </row>
     <row r="11" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -1454,30 +1466,30 @@
       <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="10"/>
       <c r="E11" s="2">
         <v>8</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G11" s="8"/>
-      <c r="H11" s="16"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="21"/>
       <c r="I11" s="2">
         <v>8</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="8"/>
-      <c r="L11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="10"/>
       <c r="M11" s="2">
         <v>8</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
-      <c r="P11" s="7"/>
+      <c r="P11" s="14"/>
       <c r="Q11" s="5" t="b">
         <v>1</v>
       </c>
@@ -1493,7 +1505,7 @@
       <c r="U11" s="1">
         <v>8</v>
       </c>
-      <c r="AF11" s="7"/>
+      <c r="AF11" s="14"/>
     </row>
     <row r="12" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -1502,32 +1514,32 @@
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="10"/>
       <c r="E12" s="2">
         <v>9</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="H12" s="16"/>
+      <c r="H12" s="21"/>
       <c r="I12" s="2">
         <v>9</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="K12" s="8"/>
-      <c r="L12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="10"/>
       <c r="M12" s="2">
         <v>9</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
-      <c r="P12" s="7"/>
+      <c r="P12" s="14"/>
       <c r="Q12" s="6" t="b">
         <v>0</v>
       </c>
@@ -1543,7 +1555,7 @@
       <c r="U12" s="1">
         <v>9</v>
       </c>
-      <c r="AF12" s="7"/>
+      <c r="AF12" s="14"/>
     </row>
     <row r="13" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
@@ -1552,34 +1564,34 @@
       <c r="B13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="9"/>
+      <c r="D13" s="10"/>
       <c r="E13" s="2">
         <v>10</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G13" s="8"/>
-      <c r="H13" s="16"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="21"/>
       <c r="I13" s="2">
         <v>10</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="K13" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="L13" s="9"/>
+      <c r="L13" s="10"/>
       <c r="M13" s="2">
         <v>10</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
-      <c r="P13" s="7"/>
+      <c r="P13" s="14"/>
       <c r="Q13" s="6" t="b">
         <v>0</v>
       </c>
@@ -1595,7 +1607,7 @@
       <c r="U13" s="1">
         <v>10</v>
       </c>
-      <c r="AF13" s="7"/>
+      <c r="AF13" s="14"/>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
@@ -1604,8 +1616,8 @@
       <c r="B14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="10"/>
       <c r="E14" s="2">
         <v>11</v>
       </c>
@@ -1615,21 +1627,21 @@
       <c r="G14" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="H14" s="16"/>
+      <c r="H14" s="21"/>
       <c r="I14" s="2">
         <v>11</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K14" s="8"/>
-      <c r="L14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="10"/>
       <c r="M14" s="2">
         <v>11</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
-      <c r="P14" s="7"/>
+      <c r="P14" s="14"/>
       <c r="Q14" s="6" t="b">
         <v>0</v>
       </c>
@@ -1645,7 +1657,7 @@
       <c r="U14" s="1">
         <v>11</v>
       </c>
-      <c r="AF14" s="7"/>
+      <c r="AF14" s="14"/>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
@@ -1654,28 +1666,28 @@
       <c r="B15" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="D15" s="9"/>
+      <c r="D15" s="10"/>
       <c r="E15" s="2">
         <v>12</v>
       </c>
-      <c r="H15" s="16"/>
+      <c r="H15" s="21"/>
       <c r="I15" s="2">
         <v>12</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="K15" s="8"/>
-      <c r="L15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="10"/>
       <c r="M15" s="2">
         <v>12</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
-      <c r="P15" s="7"/>
+      <c r="P15" s="14"/>
       <c r="Q15" s="6" t="b">
         <v>0</v>
       </c>
@@ -1691,7 +1703,7 @@
       <c r="U15" s="1">
         <v>12</v>
       </c>
-      <c r="AF15" s="7"/>
+      <c r="AF15" s="14"/>
     </row>
     <row r="16" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
@@ -1700,30 +1712,30 @@
       <c r="B16" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="10"/>
       <c r="E16" s="2">
         <v>13</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="16"/>
+      <c r="H16" s="21"/>
       <c r="I16" s="2">
         <v>13</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="K16" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L16" s="9"/>
+      <c r="L16" s="10"/>
       <c r="M16" s="2">
         <v>13</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
-      <c r="P16" s="7"/>
+      <c r="P16" s="14"/>
       <c r="Q16" s="6" t="b">
         <v>0</v>
       </c>
@@ -1739,7 +1751,7 @@
       <c r="U16" s="1">
         <v>13</v>
       </c>
-      <c r="AF16" s="7"/>
+      <c r="AF16" s="14"/>
     </row>
     <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
@@ -1748,32 +1760,32 @@
       <c r="B17" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="10"/>
       <c r="E17" s="2">
         <v>14</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="H17" s="16"/>
+      <c r="H17" s="21"/>
       <c r="I17" s="2">
         <v>14</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="K17" s="8"/>
-      <c r="L17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="10"/>
       <c r="M17" s="2">
         <v>14</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
-      <c r="P17" s="7"/>
+      <c r="P17" s="14"/>
       <c r="Q17" s="6" t="b">
         <v>0</v>
       </c>
@@ -1789,7 +1801,7 @@
       <c r="U17" s="1">
         <v>14</v>
       </c>
-      <c r="AF17" s="7"/>
+      <c r="AF17" s="14"/>
     </row>
     <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
@@ -1798,32 +1810,32 @@
       <c r="B18" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="9"/>
+      <c r="D18" s="10"/>
       <c r="E18" s="2">
         <v>15</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="G18" s="8"/>
-      <c r="H18" s="16"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="21"/>
       <c r="I18" s="2">
         <v>15</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="K18" s="8"/>
-      <c r="L18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="10"/>
       <c r="M18" s="2">
         <v>15</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
-      <c r="P18" s="7"/>
+      <c r="P18" s="14"/>
       <c r="Q18" s="6" t="b">
         <v>0</v>
       </c>
@@ -1839,7 +1851,7 @@
       <c r="U18" s="1">
         <v>15</v>
       </c>
-      <c r="AF18" s="7"/>
+      <c r="AF18" s="14"/>
     </row>
     <row r="19" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
@@ -1848,32 +1860,32 @@
       <c r="B19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="8"/>
-      <c r="D19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="10"/>
       <c r="E19" s="2">
         <v>16</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="G19" s="8"/>
-      <c r="H19" s="16"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="21"/>
       <c r="I19" s="2">
         <v>16</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="K19" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="L19" s="9"/>
+        <v>119</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="L19" s="10"/>
       <c r="M19" s="2">
         <v>16</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
-      <c r="P19" s="7"/>
+      <c r="P19" s="14"/>
       <c r="Q19" s="6" t="b">
         <v>0</v>
       </c>
@@ -1889,7 +1901,7 @@
       <c r="U19" s="1">
         <v>16</v>
       </c>
-      <c r="AF19" s="7"/>
+      <c r="AF19" s="14"/>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
@@ -1898,40 +1910,40 @@
       <c r="B20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="10"/>
       <c r="E20" s="2">
         <v>17</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="H20" s="16"/>
+      <c r="H20" s="21"/>
       <c r="I20" s="2">
         <v>17</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="K20" s="18"/>
-      <c r="L20" s="9"/>
+        <v>120</v>
+      </c>
+      <c r="K20" s="12"/>
+      <c r="L20" s="10"/>
       <c r="M20" s="2">
         <v>17</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7" t="s">
+      <c r="P20" s="14"/>
+      <c r="Q20" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="R20" s="7"/>
-      <c r="S20" s="7"/>
-      <c r="T20" s="7"/>
-      <c r="U20" s="7"/>
-      <c r="AF20" s="7"/>
+      <c r="R20" s="14"/>
+      <c r="S20" s="14"/>
+      <c r="T20" s="14"/>
+      <c r="U20" s="14"/>
+      <c r="AF20" s="14"/>
     </row>
     <row r="21" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
@@ -1940,33 +1952,33 @@
       <c r="B21" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D21" s="9"/>
+      <c r="D21" s="10"/>
       <c r="E21" s="2">
         <v>18</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G21" s="8"/>
-      <c r="H21" s="16"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="21"/>
       <c r="I21" s="2">
         <v>18</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="K21" s="19"/>
-      <c r="L21" s="9"/>
+        <v>121</v>
+      </c>
+      <c r="K21" s="13"/>
+      <c r="L21" s="10"/>
       <c r="M21" s="2">
         <v>18</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
-      <c r="P21" s="7"/>
-      <c r="AF21" s="7"/>
+      <c r="P21" s="14"/>
+      <c r="AF21" s="14"/>
     </row>
     <row r="22" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
@@ -1975,16 +1987,16 @@
       <c r="B22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="10"/>
       <c r="E22" s="2">
         <v>19</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G22" s="8"/>
-      <c r="H22" s="16"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="21"/>
       <c r="I22" s="2">
         <v>19</v>
       </c>
@@ -1994,14 +2006,14 @@
       <c r="K22" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="L22" s="9"/>
+      <c r="L22" s="10"/>
       <c r="M22" s="2">
         <v>19</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
-      <c r="P22" s="7"/>
-      <c r="AF22" s="7"/>
+      <c r="P22" s="14"/>
+      <c r="AF22" s="14"/>
     </row>
     <row r="23" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
@@ -2010,18 +2022,18 @@
       <c r="B23" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="10"/>
       <c r="E23" s="2">
         <v>20</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="H23" s="16"/>
+      <c r="H23" s="21"/>
       <c r="I23" s="2">
         <v>20</v>
       </c>
@@ -2029,30 +2041,34 @@
         <v>114</v>
       </c>
       <c r="K23" s="4"/>
-      <c r="L23" s="9"/>
+      <c r="L23" s="10"/>
       <c r="M23" s="2">
         <v>20</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
-      <c r="P23" s="7"/>
-      <c r="AF23" s="7"/>
+      <c r="P23" s="14"/>
+      <c r="AF23" s="14"/>
     </row>
     <row r="24" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>21</v>
       </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="9"/>
+      <c r="B24" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D24" s="10"/>
       <c r="E24" s="2">
         <v>21</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="G24" s="8"/>
-      <c r="H24" s="16"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="21"/>
       <c r="I24" s="2">
         <v>21</v>
       </c>
@@ -2062,74 +2078,82 @@
       <c r="K24" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="L24" s="9"/>
+      <c r="L24" s="10"/>
       <c r="M24" s="2">
         <v>21</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
-      <c r="P24" s="7"/>
-      <c r="AF24" s="7"/>
+      <c r="P24" s="14"/>
+      <c r="AF24" s="14"/>
     </row>
     <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>22</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="9"/>
+      <c r="B25" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="D25" s="10"/>
       <c r="E25" s="2">
         <v>22</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="G25" s="8"/>
-      <c r="H25" s="16"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="21"/>
       <c r="I25" s="2">
         <v>22</v>
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="4"/>
-      <c r="L25" s="9"/>
+      <c r="L25" s="10"/>
       <c r="M25" s="2">
         <v>22</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
-      <c r="P25" s="7"/>
-      <c r="AF25" s="7"/>
+      <c r="P25" s="14"/>
+      <c r="AF25" s="14"/>
     </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>23</v>
       </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="9"/>
+      <c r="B26" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="13"/>
+      <c r="D26" s="10"/>
       <c r="E26" s="2">
         <v>23</v>
       </c>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="16"/>
+      <c r="F26" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="H26" s="21"/>
       <c r="I26" s="2">
         <v>23</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="K26" s="8" t="s">
+      <c r="K26" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="L26" s="9"/>
+      <c r="L26" s="10"/>
       <c r="M26" s="2">
         <v>23</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
-      <c r="P26" s="7"/>
-      <c r="AF26" s="7"/>
+      <c r="P26" s="14"/>
+      <c r="AF26" s="14"/>
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
@@ -2138,31 +2162,33 @@
       <c r="B27" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D27" s="9"/>
+      <c r="D27" s="10"/>
       <c r="E27" s="2">
         <v>24</v>
       </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="16"/>
+      <c r="F27" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G27" s="12"/>
+      <c r="H27" s="21"/>
       <c r="I27" s="2">
         <v>24</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="K27" s="8"/>
-      <c r="L27" s="9"/>
+      <c r="K27" s="9"/>
+      <c r="L27" s="10"/>
       <c r="M27" s="2">
         <v>24</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
-      <c r="P27" s="7"/>
-      <c r="AF27" s="7"/>
+      <c r="P27" s="14"/>
+      <c r="AF27" s="14"/>
     </row>
     <row r="28" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
@@ -2171,29 +2197,31 @@
       <c r="B28" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="8"/>
-      <c r="D28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="10"/>
       <c r="E28" s="2">
         <v>25</v>
       </c>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="16"/>
+      <c r="F28" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G28" s="13"/>
+      <c r="H28" s="21"/>
       <c r="I28" s="2">
         <v>25</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="K28" s="8"/>
-      <c r="L28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="10"/>
       <c r="M28" s="2">
         <v>25</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
-      <c r="P28" s="7"/>
-      <c r="AF28" s="7"/>
+      <c r="P28" s="14"/>
+      <c r="AF28" s="14"/>
     </row>
     <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
@@ -2202,8 +2230,8 @@
       <c r="B29" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="8"/>
-      <c r="D29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="10"/>
       <c r="E29" s="2">
         <v>26</v>
       </c>
@@ -2213,7 +2241,7 @@
       <c r="G29" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H29" s="16"/>
+      <c r="H29" s="21"/>
       <c r="I29" s="2">
         <v>26</v>
       </c>
@@ -2221,14 +2249,14 @@
         <v>83</v>
       </c>
       <c r="K29" s="2"/>
-      <c r="L29" s="9"/>
+      <c r="L29" s="10"/>
       <c r="M29" s="2">
         <v>26</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
-      <c r="P29" s="7"/>
-      <c r="AF29" s="7"/>
+      <c r="P29" s="14"/>
+      <c r="AF29" s="14"/>
     </row>
     <row r="30" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
@@ -2238,13 +2266,13 @@
         <v>99</v>
       </c>
       <c r="C30" s="2"/>
-      <c r="D30" s="9"/>
+      <c r="D30" s="10"/>
       <c r="E30" s="2">
         <v>27</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
-      <c r="H30" s="16"/>
+      <c r="H30" s="21"/>
       <c r="I30" s="2">
         <v>27</v>
       </c>
@@ -2252,14 +2280,14 @@
         <v>113</v>
       </c>
       <c r="K30" s="2"/>
-      <c r="L30" s="9"/>
+      <c r="L30" s="10"/>
       <c r="M30" s="2">
         <v>27</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
-      <c r="P30" s="7"/>
-      <c r="AF30" s="7"/>
+      <c r="P30" s="14"/>
+      <c r="AF30" s="14"/>
     </row>
     <row r="31" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
@@ -2269,7 +2297,7 @@
         <v>98</v>
       </c>
       <c r="C31" s="2"/>
-      <c r="D31" s="9"/>
+      <c r="D31" s="10"/>
       <c r="E31" s="2">
         <v>28</v>
       </c>
@@ -2279,7 +2307,7 @@
       <c r="G31" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H31" s="16"/>
+      <c r="H31" s="21"/>
       <c r="I31" s="2">
         <v>28</v>
       </c>
@@ -2287,14 +2315,14 @@
         <v>77</v>
       </c>
       <c r="K31" s="2"/>
-      <c r="L31" s="9"/>
+      <c r="L31" s="10"/>
       <c r="M31" s="2">
         <v>28</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
-      <c r="P31" s="7"/>
-      <c r="AF31" s="7"/>
+      <c r="P31" s="14"/>
+      <c r="AF31" s="14"/>
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
@@ -2302,13 +2330,13 @@
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="9"/>
+      <c r="D32" s="10"/>
       <c r="E32" s="2">
         <v>29</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
-      <c r="H32" s="16"/>
+      <c r="H32" s="21"/>
       <c r="I32" s="2">
         <v>29</v>
       </c>
@@ -2318,14 +2346,14 @@
       <c r="K32" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="L32" s="9"/>
+      <c r="L32" s="10"/>
       <c r="M32" s="2">
         <v>29</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
-      <c r="P32" s="7"/>
-      <c r="AF32" s="7"/>
+      <c r="P32" s="14"/>
+      <c r="AF32" s="14"/>
     </row>
     <row r="33" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
@@ -2334,20 +2362,20 @@
       <c r="B33" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="C33" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="10"/>
       <c r="E33" s="2">
         <v>30</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G33" s="8" t="s">
+      <c r="G33" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="16"/>
+      <c r="H33" s="21"/>
       <c r="I33" s="2">
         <v>30</v>
       </c>
@@ -2355,14 +2383,14 @@
         <v>84</v>
       </c>
       <c r="K33" s="2"/>
-      <c r="L33" s="9"/>
+      <c r="L33" s="10"/>
       <c r="M33" s="2">
         <v>30</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
-      <c r="P33" s="7"/>
-      <c r="AF33" s="7"/>
+      <c r="P33" s="14"/>
+      <c r="AF33" s="14"/>
     </row>
     <row r="34" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
@@ -2371,16 +2399,16 @@
       <c r="B34" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C34" s="18"/>
-      <c r="D34" s="9"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="10"/>
       <c r="E34" s="2">
         <v>31</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="G34" s="8"/>
-      <c r="H34" s="16"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="21"/>
       <c r="I34" s="2">
         <v>31</v>
       </c>
@@ -2388,14 +2416,14 @@
         <v>95</v>
       </c>
       <c r="K34" s="2"/>
-      <c r="L34" s="9"/>
+      <c r="L34" s="10"/>
       <c r="M34" s="2">
         <v>31</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
-      <c r="P34" s="7"/>
-      <c r="AF34" s="7"/>
+      <c r="P34" s="14"/>
+      <c r="AF34" s="14"/>
     </row>
     <row r="35" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
@@ -2404,16 +2432,16 @@
       <c r="B35" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C35" s="19"/>
-      <c r="D35" s="9"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="10"/>
       <c r="E35" s="2">
         <v>32</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G35" s="8"/>
-      <c r="H35" s="16"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="21"/>
       <c r="I35" s="2">
         <v>32</v>
       </c>
@@ -2421,77 +2449,77 @@
         <v>115</v>
       </c>
       <c r="K35" s="2"/>
-      <c r="L35" s="9"/>
+      <c r="L35" s="10"/>
       <c r="M35" s="2">
         <v>32</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
-      <c r="P35" s="7"/>
-      <c r="AF35" s="7"/>
+      <c r="P35" s="14"/>
+      <c r="AF35" s="14"/>
     </row>
     <row r="36" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A36" s="10"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="11"/>
-      <c r="K36" s="11"/>
-      <c r="L36" s="11"/>
-      <c r="M36" s="11"/>
-      <c r="N36" s="11"/>
-      <c r="O36" s="12"/>
+      <c r="A36" s="15"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="16"/>
+      <c r="L36" s="16"/>
+      <c r="M36" s="16"/>
+      <c r="N36" s="16"/>
+      <c r="O36" s="17"/>
     </row>
     <row r="37" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="9" t="s">
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="J37" s="9"/>
-      <c r="K37" s="9"/>
-      <c r="L37" s="9"/>
-      <c r="M37" s="9"/>
-      <c r="N37" s="9"/>
-      <c r="O37" s="9"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+      <c r="N37" s="10"/>
+      <c r="O37" s="10"/>
     </row>
     <row r="38" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
+      <c r="A38" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9" t="s">
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="9" t="s">
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="J38" s="9"/>
-      <c r="K38" s="9"/>
-      <c r="L38" s="9"/>
-      <c r="M38" s="9" t="s">
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="N38" s="9"/>
-      <c r="O38" s="9"/>
+      <c r="N38" s="10"/>
+      <c r="O38" s="10"/>
     </row>
     <row r="39" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
@@ -2503,7 +2531,7 @@
       <c r="C39" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D39" s="9"/>
+      <c r="D39" s="10"/>
       <c r="E39" s="3" t="s">
         <v>0</v>
       </c>
@@ -2513,7 +2541,7 @@
       <c r="G39" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H39" s="14"/>
+      <c r="H39" s="19"/>
       <c r="I39" s="3" t="s">
         <v>0</v>
       </c>
@@ -2523,7 +2551,7 @@
       <c r="K39" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="L39" s="9"/>
+      <c r="L39" s="10"/>
       <c r="M39" s="3" t="s">
         <v>0</v>
       </c>
@@ -2541,26 +2569,26 @@
       <c r="B40" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D40" s="9"/>
+      <c r="D40" s="10"/>
       <c r="E40" s="2">
         <v>1</v>
       </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
-      <c r="H40" s="14"/>
+      <c r="H40" s="19"/>
       <c r="I40" s="2">
         <v>1</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="K40" s="8" t="s">
+      <c r="K40" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="L40" s="9"/>
+      <c r="L40" s="10"/>
       <c r="M40" s="2">
         <v>1</v>
       </c>
@@ -2574,22 +2602,22 @@
       <c r="B41" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C41" s="8"/>
-      <c r="D41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="10"/>
       <c r="E41" s="2">
         <v>2</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
-      <c r="H41" s="14"/>
+      <c r="H41" s="19"/>
       <c r="I41" s="2">
         <v>2</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K41" s="8"/>
-      <c r="L41" s="9"/>
+      <c r="K41" s="9"/>
+      <c r="L41" s="10"/>
       <c r="M41" s="2">
         <v>2</v>
       </c>
@@ -2603,22 +2631,22 @@
       <c r="B42" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="10"/>
       <c r="E42" s="2">
         <v>3</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
-      <c r="H42" s="14"/>
+      <c r="H42" s="19"/>
       <c r="I42" s="2">
         <v>3</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K42" s="8"/>
-      <c r="L42" s="9"/>
+      <c r="K42" s="9"/>
+      <c r="L42" s="10"/>
       <c r="M42" s="2">
         <v>3</v>
       </c>
@@ -2632,24 +2660,24 @@
       <c r="B43" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C43" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D43" s="9"/>
+      <c r="D43" s="10"/>
       <c r="E43" s="2">
         <v>4</v>
       </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
-      <c r="H43" s="14"/>
+      <c r="H43" s="19"/>
       <c r="I43" s="2">
         <v>4</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="K43" s="8"/>
-      <c r="L43" s="9"/>
+      <c r="K43" s="9"/>
+      <c r="L43" s="10"/>
       <c r="M43" s="2">
         <v>4</v>
       </c>
@@ -2663,22 +2691,22 @@
       <c r="B44" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="10"/>
       <c r="E44" s="2">
         <v>5</v>
       </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
-      <c r="H44" s="14"/>
+      <c r="H44" s="19"/>
       <c r="I44" s="2">
         <v>5</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K44" s="8"/>
-      <c r="L44" s="9"/>
+      <c r="K44" s="9"/>
+      <c r="L44" s="10"/>
       <c r="M44" s="2">
         <v>5</v>
       </c>
@@ -2692,22 +2720,22 @@
       <c r="B45" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C45" s="8"/>
-      <c r="D45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="10"/>
       <c r="E45" s="2">
         <v>6</v>
       </c>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
-      <c r="H45" s="14"/>
+      <c r="H45" s="19"/>
       <c r="I45" s="2">
         <v>6</v>
       </c>
       <c r="J45" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K45" s="8"/>
-      <c r="L45" s="9"/>
+      <c r="K45" s="9"/>
+      <c r="L45" s="10"/>
       <c r="M45" s="2">
         <v>6</v>
       </c>
@@ -2721,24 +2749,24 @@
       <c r="B46" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C46" s="8" t="s">
+      <c r="C46" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D46" s="9"/>
+      <c r="D46" s="10"/>
       <c r="E46" s="2">
         <v>7</v>
       </c>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
-      <c r="H46" s="14"/>
+      <c r="H46" s="19"/>
       <c r="I46" s="2">
         <v>7</v>
       </c>
       <c r="J46" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="K46" s="8"/>
-      <c r="L46" s="9"/>
+      <c r="K46" s="9"/>
+      <c r="L46" s="10"/>
       <c r="M46" s="2">
         <v>7</v>
       </c>
@@ -2752,22 +2780,22 @@
       <c r="B47" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C47" s="8"/>
-      <c r="D47" s="9"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="10"/>
       <c r="E47" s="2">
         <v>8</v>
       </c>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
-      <c r="H47" s="14"/>
+      <c r="H47" s="19"/>
       <c r="I47" s="2">
         <v>8</v>
       </c>
       <c r="J47" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K47" s="8"/>
-      <c r="L47" s="9"/>
+      <c r="K47" s="9"/>
+      <c r="L47" s="10"/>
       <c r="M47" s="2">
         <v>8</v>
       </c>
@@ -2781,22 +2809,22 @@
       <c r="B48" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C48" s="8"/>
-      <c r="D48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="10"/>
       <c r="E48" s="2">
         <v>9</v>
       </c>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
-      <c r="H48" s="14"/>
+      <c r="H48" s="19"/>
       <c r="I48" s="2">
         <v>9</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K48" s="8"/>
-      <c r="L48" s="9"/>
+      <c r="K48" s="9"/>
+      <c r="L48" s="10"/>
       <c r="M48" s="2">
         <v>9</v>
       </c>
@@ -2810,24 +2838,24 @@
       <c r="B49" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="C49" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D49" s="9"/>
+      <c r="D49" s="10"/>
       <c r="E49" s="2">
         <v>10</v>
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="2"/>
-      <c r="H49" s="14"/>
+      <c r="H49" s="19"/>
       <c r="I49" s="2">
         <v>10</v>
       </c>
       <c r="J49" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="K49" s="8"/>
-      <c r="L49" s="9"/>
+      <c r="K49" s="9"/>
+      <c r="L49" s="10"/>
       <c r="M49" s="2">
         <v>10</v>
       </c>
@@ -2841,22 +2869,22 @@
       <c r="B50" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="10"/>
       <c r="E50" s="2">
         <v>11</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
-      <c r="H50" s="14"/>
+      <c r="H50" s="19"/>
       <c r="I50" s="2">
         <v>11</v>
       </c>
       <c r="J50" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="K50" s="8"/>
-      <c r="L50" s="9"/>
+      <c r="K50" s="9"/>
+      <c r="L50" s="10"/>
       <c r="M50" s="2">
         <v>11</v>
       </c>
@@ -2870,22 +2898,22 @@
       <c r="B51" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C51" s="8"/>
-      <c r="D51" s="9"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="10"/>
       <c r="E51" s="2">
         <v>12</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="2"/>
-      <c r="H51" s="14"/>
+      <c r="H51" s="19"/>
       <c r="I51" s="2">
         <v>12</v>
       </c>
       <c r="J51" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="K51" s="8"/>
-      <c r="L51" s="9"/>
+      <c r="K51" s="9"/>
+      <c r="L51" s="10"/>
       <c r="M51" s="2">
         <v>12</v>
       </c>
@@ -2899,26 +2927,26 @@
       <c r="B52" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C52" s="8" t="s">
+      <c r="C52" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D52" s="9"/>
+      <c r="D52" s="10"/>
       <c r="E52" s="2">
         <v>13</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
-      <c r="H52" s="14"/>
+      <c r="H52" s="19"/>
       <c r="I52" s="2">
         <v>13</v>
       </c>
       <c r="J52" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="K52" s="8" t="s">
+      <c r="K52" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="L52" s="9"/>
+      <c r="L52" s="10"/>
       <c r="M52" s="2">
         <v>13</v>
       </c>
@@ -2932,22 +2960,22 @@
       <c r="B53" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="10"/>
       <c r="E53" s="2">
         <v>14</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
-      <c r="H53" s="14"/>
+      <c r="H53" s="19"/>
       <c r="I53" s="2">
         <v>14</v>
       </c>
       <c r="J53" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K53" s="8"/>
-      <c r="L53" s="9"/>
+      <c r="K53" s="9"/>
+      <c r="L53" s="10"/>
       <c r="M53" s="2">
         <v>14</v>
       </c>
@@ -2961,22 +2989,22 @@
       <c r="B54" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="10"/>
       <c r="E54" s="2">
         <v>15</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
-      <c r="H54" s="14"/>
+      <c r="H54" s="19"/>
       <c r="I54" s="2">
         <v>15</v>
       </c>
       <c r="J54" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="K54" s="8"/>
-      <c r="L54" s="9"/>
+      <c r="K54" s="9"/>
+      <c r="L54" s="10"/>
       <c r="M54" s="2">
         <v>15</v>
       </c>
@@ -2989,13 +3017,13 @@
       </c>
       <c r="B55" s="2"/>
       <c r="C55" s="4"/>
-      <c r="D55" s="9"/>
+      <c r="D55" s="10"/>
       <c r="E55" s="2">
         <v>16</v>
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
-      <c r="H55" s="14"/>
+      <c r="H55" s="19"/>
       <c r="I55" s="2">
         <v>16</v>
       </c>
@@ -3005,7 +3033,7 @@
       <c r="K55" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="L55" s="9"/>
+      <c r="L55" s="10"/>
       <c r="M55" s="2">
         <v>16</v>
       </c>
@@ -3018,13 +3046,13 @@
       </c>
       <c r="B56" s="2"/>
       <c r="C56" s="4"/>
-      <c r="D56" s="9"/>
+      <c r="D56" s="10"/>
       <c r="E56" s="2">
         <v>17</v>
       </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
-      <c r="H56" s="14"/>
+      <c r="H56" s="19"/>
       <c r="I56" s="2">
         <v>17</v>
       </c>
@@ -3032,7 +3060,7 @@
         <v>77</v>
       </c>
       <c r="K56" s="2"/>
-      <c r="L56" s="9"/>
+      <c r="L56" s="10"/>
       <c r="M56" s="2">
         <v>17</v>
       </c>
@@ -3045,13 +3073,13 @@
       </c>
       <c r="B57" s="2"/>
       <c r="C57" s="4"/>
-      <c r="D57" s="9"/>
+      <c r="D57" s="10"/>
       <c r="E57" s="2">
         <v>18</v>
       </c>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
-      <c r="H57" s="14"/>
+      <c r="H57" s="19"/>
       <c r="I57" s="2">
         <v>18</v>
       </c>
@@ -3059,7 +3087,7 @@
         <v>83</v>
       </c>
       <c r="K57" s="2"/>
-      <c r="L57" s="9"/>
+      <c r="L57" s="10"/>
       <c r="M57" s="2">
         <v>18</v>
       </c>
@@ -3073,16 +3101,16 @@
       <c r="B58" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C58" s="8" t="s">
+      <c r="C58" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D58" s="9"/>
+      <c r="D58" s="10"/>
       <c r="E58" s="2">
         <v>19</v>
       </c>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
-      <c r="H58" s="14"/>
+      <c r="H58" s="19"/>
       <c r="I58" s="2">
         <v>19</v>
       </c>
@@ -3092,7 +3120,7 @@
       <c r="K58" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="L58" s="9"/>
+      <c r="L58" s="10"/>
       <c r="M58" s="2">
         <v>19</v>
       </c>
@@ -3104,14 +3132,14 @@
         <v>20</v>
       </c>
       <c r="B59" s="2"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="10"/>
       <c r="E59" s="2">
         <v>20</v>
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
-      <c r="H59" s="14"/>
+      <c r="H59" s="19"/>
       <c r="I59" s="2">
         <v>20</v>
       </c>
@@ -3119,7 +3147,7 @@
         <v>81</v>
       </c>
       <c r="K59" s="2"/>
-      <c r="L59" s="9"/>
+      <c r="L59" s="10"/>
       <c r="M59" s="2">
         <v>20</v>
       </c>
@@ -3133,20 +3161,20 @@
       <c r="B60" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C60" s="8"/>
-      <c r="D60" s="9"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="10"/>
       <c r="E60" s="2">
         <v>21</v>
       </c>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
-      <c r="H60" s="14"/>
+      <c r="H60" s="19"/>
       <c r="I60" s="2">
         <v>21</v>
       </c>
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
-      <c r="L60" s="9"/>
+      <c r="L60" s="10"/>
       <c r="M60" s="2">
         <v>21</v>
       </c>
@@ -3158,20 +3186,20 @@
         <v>22</v>
       </c>
       <c r="B61" s="2"/>
-      <c r="C61" s="8"/>
-      <c r="D61" s="9"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="10"/>
       <c r="E61" s="2">
         <v>22</v>
       </c>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
-      <c r="H61" s="14"/>
+      <c r="H61" s="19"/>
       <c r="I61" s="2">
         <v>22</v>
       </c>
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
-      <c r="L61" s="9"/>
+      <c r="L61" s="10"/>
       <c r="M61" s="2">
         <v>22</v>
       </c>
@@ -3188,19 +3216,19 @@
       <c r="C62" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D62" s="9"/>
+      <c r="D62" s="10"/>
       <c r="E62" s="2">
         <v>23</v>
       </c>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
-      <c r="H62" s="14"/>
+      <c r="H62" s="19"/>
       <c r="I62" s="2">
         <v>23</v>
       </c>
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
-      <c r="L62" s="9"/>
+      <c r="L62" s="10"/>
       <c r="M62" s="2">
         <v>23</v>
       </c>
@@ -3215,19 +3243,19 @@
         <v>60</v>
       </c>
       <c r="C63" s="2"/>
-      <c r="D63" s="9"/>
+      <c r="D63" s="10"/>
       <c r="E63" s="2">
         <v>24</v>
       </c>
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
-      <c r="H63" s="14"/>
+      <c r="H63" s="19"/>
       <c r="I63" s="2">
         <v>24</v>
       </c>
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
-      <c r="L63" s="9"/>
+      <c r="L63" s="10"/>
       <c r="M63" s="2">
         <v>24</v>
       </c>
@@ -3242,19 +3270,19 @@
         <v>61</v>
       </c>
       <c r="C64" s="2"/>
-      <c r="D64" s="9"/>
+      <c r="D64" s="10"/>
       <c r="E64" s="2">
         <v>25</v>
       </c>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
-      <c r="H64" s="14"/>
+      <c r="H64" s="19"/>
       <c r="I64" s="2">
         <v>25</v>
       </c>
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
-      <c r="L64" s="9"/>
+      <c r="L64" s="10"/>
       <c r="M64" s="2">
         <v>25</v>
       </c>
@@ -3271,19 +3299,19 @@
       <c r="C65" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D65" s="9"/>
+      <c r="D65" s="10"/>
       <c r="E65" s="2">
         <v>26</v>
       </c>
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
-      <c r="H65" s="14"/>
+      <c r="H65" s="19"/>
       <c r="I65" s="2">
         <v>26</v>
       </c>
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
-      <c r="L65" s="9"/>
+      <c r="L65" s="10"/>
       <c r="M65" s="2">
         <v>26</v>
       </c>
@@ -3298,19 +3326,19 @@
         <v>95</v>
       </c>
       <c r="C66" s="2"/>
-      <c r="D66" s="9"/>
+      <c r="D66" s="10"/>
       <c r="E66" s="2">
         <v>27</v>
       </c>
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
-      <c r="H66" s="14"/>
+      <c r="H66" s="19"/>
       <c r="I66" s="2">
         <v>27</v>
       </c>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
-      <c r="L66" s="9"/>
+      <c r="L66" s="10"/>
       <c r="M66" s="2">
         <v>27</v>
       </c>
@@ -3325,19 +3353,19 @@
         <v>97</v>
       </c>
       <c r="C67" s="2"/>
-      <c r="D67" s="9"/>
+      <c r="D67" s="10"/>
       <c r="E67" s="2">
         <v>28</v>
       </c>
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
-      <c r="H67" s="14"/>
+      <c r="H67" s="19"/>
       <c r="I67" s="2">
         <v>28</v>
       </c>
       <c r="J67" s="2"/>
       <c r="K67" s="2"/>
-      <c r="L67" s="9"/>
+      <c r="L67" s="10"/>
       <c r="M67" s="2">
         <v>28</v>
       </c>
@@ -3350,19 +3378,19 @@
       </c>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
-      <c r="D68" s="9"/>
+      <c r="D68" s="10"/>
       <c r="E68" s="2">
         <v>29</v>
       </c>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
-      <c r="H68" s="14"/>
+      <c r="H68" s="19"/>
       <c r="I68" s="2">
         <v>29</v>
       </c>
       <c r="J68" s="2"/>
       <c r="K68" s="2"/>
-      <c r="L68" s="9"/>
+      <c r="L68" s="10"/>
       <c r="M68" s="2">
         <v>29</v>
       </c>
@@ -3375,19 +3403,19 @@
       </c>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
-      <c r="D69" s="9"/>
+      <c r="D69" s="10"/>
       <c r="E69" s="2">
         <v>30</v>
       </c>
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
-      <c r="H69" s="14"/>
+      <c r="H69" s="19"/>
       <c r="I69" s="2">
         <v>30</v>
       </c>
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
-      <c r="L69" s="9"/>
+      <c r="L69" s="10"/>
       <c r="M69" s="2">
         <v>30</v>
       </c>
@@ -3400,19 +3428,19 @@
       </c>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
-      <c r="D70" s="9"/>
+      <c r="D70" s="10"/>
       <c r="E70" s="2">
         <v>31</v>
       </c>
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
-      <c r="H70" s="14"/>
+      <c r="H70" s="19"/>
       <c r="I70" s="2">
         <v>31</v>
       </c>
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
-      <c r="L70" s="9"/>
+      <c r="L70" s="10"/>
       <c r="M70" s="2">
         <v>31</v>
       </c>
@@ -3425,19 +3453,19 @@
       </c>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
-      <c r="D71" s="9"/>
+      <c r="D71" s="10"/>
       <c r="E71" s="2">
         <v>32</v>
       </c>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
-      <c r="H71" s="15"/>
+      <c r="H71" s="20"/>
       <c r="I71" s="2">
         <v>32</v>
       </c>
       <c r="J71" s="2"/>
       <c r="K71" s="2"/>
-      <c r="L71" s="9"/>
+      <c r="L71" s="10"/>
       <c r="M71" s="2">
         <v>32</v>
       </c>
@@ -3445,12 +3473,19 @@
       <c r="O71" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="54">
-    <mergeCell ref="C33:C35"/>
-    <mergeCell ref="Q20:U20"/>
+  <mergeCells count="56">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="G4:G5"/>
+    <mergeCell ref="G17:G19"/>
+    <mergeCell ref="G33:G35"/>
+    <mergeCell ref="K26:K28"/>
+    <mergeCell ref="C33:C35"/>
+    <mergeCell ref="Q20:U20"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="C40:C42"/>
     <mergeCell ref="AF1:AF35"/>
     <mergeCell ref="P1:P35"/>
     <mergeCell ref="H1:H35"/>
@@ -3461,6 +3496,12 @@
     <mergeCell ref="C21:C23"/>
     <mergeCell ref="C18:C20"/>
     <mergeCell ref="C15:C17"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="D2:D35"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="Q1:U1"/>
     <mergeCell ref="K40:K51"/>
     <mergeCell ref="A36:O36"/>
     <mergeCell ref="H37:H71"/>
@@ -3469,24 +3510,10 @@
     <mergeCell ref="L38:L71"/>
     <mergeCell ref="M38:O38"/>
     <mergeCell ref="K52:K54"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="G17:G19"/>
-    <mergeCell ref="G33:G35"/>
-    <mergeCell ref="K26:K28"/>
     <mergeCell ref="A37:G37"/>
     <mergeCell ref="A38:C38"/>
     <mergeCell ref="D38:D71"/>
     <mergeCell ref="E38:G38"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="D2:D35"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="Q1:U1"/>
     <mergeCell ref="C52:C54"/>
     <mergeCell ref="G20:G22"/>
     <mergeCell ref="G23:G25"/>
@@ -3499,7 +3526,10 @@
     <mergeCell ref="K10:K12"/>
     <mergeCell ref="K13:K15"/>
     <mergeCell ref="K16:K18"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="G26:G28"/>
     <mergeCell ref="K19:K21"/>
+    <mergeCell ref="C43:C45"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>